<commit_message>
report: update 2026-04-05 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2527,7 +2527,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M159"/>
+  <dimension ref="A1:M199"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46115</v>
+        <v>46117</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D28" s="36" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发1次</t>
+          <t>累计未发1次，迟发2次</t>
         </is>
       </c>
     </row>
@@ -3927,6 +3927,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
     </row>
     <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
@@ -3942,6 +3947,11 @@
       <c r="C56" s="60" t="inlineStr">
         <is>
           <t>是</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
         </is>
       </c>
     </row>
@@ -4064,6 +4074,46 @@
     <row r="157"/>
     <row r="158"/>
     <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
report: update 2026-04-06 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2527,7 +2527,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M199"/>
+  <dimension ref="A1:M219"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46117</v>
+        <v>46118</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3313,7 +3313,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D26" s="33" t="n"/>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
     </row>
     <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
@@ -3355,7 +3359,7 @@
       </c>
       <c r="D28" s="36" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发2次</t>
+          <t>累计未发1次，迟发3次</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3785,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D48" s="36" t="n"/>
+      <c r="D48" s="36" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
     </row>
     <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
@@ -3927,7 +3935,7 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="0" t="inlineStr">
         <is>
           <t>累计未发1次</t>
         </is>
@@ -3949,7 +3957,7 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="0" t="inlineStr">
         <is>
           <t>累计未发1次</t>
         </is>
@@ -4114,6 +4122,26 @@
     <row r="197"/>
     <row r="198"/>
     <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
report: update 2026-04-07 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2527,7 +2527,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M219"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3918,6 +3918,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
     </row>
     <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
@@ -3980,168 +3985,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
report: update 2026-04-09 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2544,7 +2544,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46119</v>
+        <v>46121</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="D34" s="36" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发4次</t>
+          <t>累计未发2次，迟发5次</t>
         </is>
       </c>
     </row>
@@ -3918,7 +3918,7 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="0" t="inlineStr">
         <is>
           <t>累计未发1次</t>
         </is>

</xml_diff>

<commit_message>
report: update 2026-04-11 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46122</v>
+        <v>46123</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="D52" s="73" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E52" s="72" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-04-14 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46123</v>
+        <v>46126</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="D24" s="74" t="inlineStr">
         <is>
-          <t>累计迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E24" s="72" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-04-15 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2612,7 +2612,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O259"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="D49" s="74" t="inlineStr">
         <is>
-          <t>累计迟发1次</t>
+          <t>累计迟发2次</t>
         </is>
       </c>
       <c r="E49" s="72" t="n"/>
@@ -4400,7 +4400,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D54" s="71" t="n"/>
+      <c r="D54" s="71" t="inlineStr">
+        <is>
+          <t>累计迟发1次</t>
+        </is>
+      </c>
       <c r="E54" s="72" t="n"/>
       <c r="F54" s="79" t="inlineStr">
         <is>
@@ -4509,6 +4513,207 @@
       </c>
       <c r="G58" s="70" t="n"/>
     </row>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
   </sheetData>
   <autoFilter ref="A2:F58"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
report: update 2026-04-17 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2632,7 +2632,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2995,7 +2995,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D8" s="68" t="n"/>
+      <c r="D8" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E8" s="69" t="n"/>
       <c r="F8" s="63" t="inlineStr">
         <is>
@@ -3083,7 +3087,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D10" s="70" t="n"/>
+      <c r="D10" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E10" s="69" t="n"/>
       <c r="F10" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-04-19 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2632,7 +2632,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46129</v>
+        <v>46131</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D7" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发3次</t>
+          <t>累计未发2次，迟发3次</t>
         </is>
       </c>
       <c r="E7" s="69" t="n"/>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="D42" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E42" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-04-20 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2615,7 +2615,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O259"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2632,7 +2632,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46131</v>
+        <v>46132</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="D15" s="70" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发1次</t>
+          <t>累计未发2次，迟发2次</t>
         </is>
       </c>
       <c r="E15" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-04-21 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2615,7 +2615,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:O259"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2632,7 +2632,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="D8" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E8" s="69" t="n"/>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E10" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-04-26 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2612,7 +2612,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O299"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46136</v>
+        <v>46138</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="D46" s="71" t="inlineStr">
         <is>
-          <t>累计迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E46" s="69" t="n"/>
@@ -4207,7 +4207,7 @@
       </c>
       <c r="D47" s="71" t="inlineStr">
         <is>
-          <t>累计迟发2次</t>
+          <t>累计未发1次，迟发2次</t>
         </is>
       </c>
       <c r="E47" s="69" t="n"/>
@@ -4236,7 +4236,7 @@
       </c>
       <c r="D48" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E48" s="69" t="n"/>
@@ -4768,6 +4768,46 @@
     <row customHeight="1" ht="16" r="257" s="53"/>
     <row customHeight="1" ht="16" r="258" s="53"/>
     <row customHeight="1" ht="16" r="259" s="53"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
   </sheetData>
   <autoFilter ref="A2:F58"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
report: update 2026-04-27 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2612,7 +2612,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O299"/>
+  <dimension ref="A1:O319"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46138</v>
+        <v>46139</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="D33" s="73" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发1次</t>
+          <t>累计未发2次，迟发2次</t>
         </is>
       </c>
       <c r="E33" s="69" t="n"/>
@@ -4097,7 +4097,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D43" s="71" t="n"/>
+      <c r="D43" s="71" t="inlineStr">
+        <is>
+          <t>累计迟发1次</t>
+        </is>
+      </c>
       <c r="E43" s="69" t="n"/>
       <c r="F43" s="63" t="inlineStr">
         <is>
@@ -4808,6 +4812,26 @@
     <row r="297"/>
     <row r="298"/>
     <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
   </sheetData>
   <autoFilter ref="A2:F58"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
report: update 2026-04-30 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2612,7 +2612,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O319"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
     <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46139</v>
+        <v>46142</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="D8" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E8" s="69" t="n"/>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E10" s="69" t="n"/>
@@ -3817,7 +3817,7 @@
       </c>
       <c r="D33" s="73" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发2次</t>
+          <t>累计未发2次，迟发3次</t>
         </is>
       </c>
       <c r="E33" s="69" t="n"/>
@@ -4772,66 +4772,6 @@
     <row customHeight="1" ht="16" r="257" s="53"/>
     <row customHeight="1" ht="16" r="258" s="53"/>
     <row customHeight="1" ht="16" r="259" s="53"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
   </sheetData>
   <autoFilter ref="A2:F58"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
report: update 2026-05-02 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46142</v>
+        <v>46144</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="D6" s="68" t="inlineStr">
         <is>
-          <t>累计未发4次</t>
+          <t>累计未发5次</t>
         </is>
       </c>
       <c r="E6" s="69" t="n"/>
@@ -2994,7 +2994,7 @@
       </c>
       <c r="D8" s="68" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发4次</t>
         </is>
       </c>
       <c r="E8" s="69" t="n"/>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发4次</t>
         </is>
       </c>
       <c r="E10" s="69" t="n"/>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="D27" s="68" t="inlineStr">
         <is>
-          <t>累计未发5次，迟发1次</t>
+          <t>累计未发6次，迟发1次</t>
         </is>
       </c>
       <c r="E27" s="69" t="n"/>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="D32" s="71" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发2次</t>
+          <t>累计未发4次，迟发2次</t>
         </is>
       </c>
       <c r="E32" s="69" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="D42" s="71" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E42" s="69" t="n"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="D50" s="70" t="inlineStr">
         <is>
-          <t>累计迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E50" s="69" t="n"/>
@@ -4327,7 +4327,7 @@
       </c>
       <c r="D51" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E51" s="69" t="n"/>
@@ -4441,7 +4441,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D55" s="68" t="n"/>
+      <c r="D55" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E55" s="69" t="n"/>
       <c r="F55" s="63" t="inlineStr">
         <is>
@@ -4491,7 +4495,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D57" s="68" t="n"/>
+      <c r="D57" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E57" s="69" t="n"/>
       <c r="F57" s="63" t="inlineStr">
         <is>
@@ -4541,7 +4549,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D59" s="68" t="n"/>
+      <c r="D59" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E59" s="69" t="n"/>
       <c r="F59" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-05-03 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46144</v>
+        <v>46145</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="D48" s="71" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E48" s="69" t="n"/>
@@ -4470,7 +4470,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D56" s="68" t="n"/>
+      <c r="D56" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E56" s="69" t="n"/>
       <c r="F56" s="63" t="inlineStr">
         <is>
@@ -4497,7 +4501,7 @@
       </c>
       <c r="D57" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E57" s="69" t="n"/>
@@ -4524,7 +4528,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D58" s="68" t="n"/>
+      <c r="D58" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E58" s="69" t="n"/>
       <c r="F58" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-05-04 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46145</v>
+        <v>46146</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3784,7 +3784,7 @@
       </c>
       <c r="D32" s="71" t="inlineStr">
         <is>
-          <t>累计未发4次，迟发2次</t>
+          <t>累计未发4次，迟发3次</t>
         </is>
       </c>
       <c r="E32" s="69" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="D36" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发2次</t>
+          <t>累计未发1次，迟发3次</t>
         </is>
       </c>
       <c r="E36" s="69" t="n"/>
@@ -4153,7 +4153,7 @@
       </c>
       <c r="D45" s="71" t="inlineStr">
         <is>
-          <t>累计迟发2次</t>
+          <t>迟发3次</t>
         </is>
       </c>
       <c r="E45" s="69" t="n"/>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="D55" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="D57" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发2次，迟发1次</t>
         </is>
       </c>
       <c r="E57" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-05 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="D15" s="70" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发2次</t>
+          <t>累计未发3次，迟发2次</t>
         </is>
       </c>
       <c r="E15" s="69" t="n"/>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="D27" s="68" t="inlineStr">
         <is>
-          <t>累计未发6次，迟发1次</t>
+          <t>累计未发7次，迟发1次</t>
         </is>
       </c>
       <c r="E27" s="69" t="n"/>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="D32" s="71" t="inlineStr">
         <is>
-          <t>累计未发4次，迟发3次</t>
+          <t>累计未发5次，迟发3次</t>
         </is>
       </c>
       <c r="E32" s="69" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="D58" s="68" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>迟发2次</t>
         </is>
       </c>
       <c r="E58" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-06 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46147</v>
+        <v>46148</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="D21" s="70" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发2次</t>
+          <t>累计未发3次，迟发2次</t>
         </is>
       </c>
       <c r="E21" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-10 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46148</v>
+        <v>46152</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="D13" s="70" t="inlineStr">
         <is>
-          <t>累计未发4次</t>
+          <t>累计未发4次，迟发1次</t>
         </is>
       </c>
       <c r="E13" s="70" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-11 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="D48" s="71" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发4次</t>
         </is>
       </c>
       <c r="E48" s="69" t="n"/>
@@ -4530,7 +4530,7 @@
       </c>
       <c r="D58" s="68" t="inlineStr">
         <is>
-          <t>迟发2次</t>
+          <t>迟发3次</t>
         </is>
       </c>
       <c r="E58" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-12 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="D24" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发1次</t>
+          <t>累计未发2次，迟发1次</t>
         </is>
       </c>
       <c r="E24" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-13 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="D27" s="68" t="inlineStr">
         <is>
-          <t>累计未发7次，迟发1次</t>
+          <t>累计未发8次，迟发1次</t>
         </is>
       </c>
       <c r="E27" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-14 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3172,7 +3172,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D12" s="73" t="n"/>
+      <c r="D12" s="73" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E12" s="69" t="n"/>
       <c r="F12" s="63" t="inlineStr">
         <is>
@@ -3390,7 +3394,7 @@
       </c>
       <c r="D18" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E18" s="69" t="n"/>
@@ -4070,7 +4074,7 @@
       </c>
       <c r="D42" s="71" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发4次</t>
         </is>
       </c>
       <c r="E42" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-17 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46156</v>
+        <v>46159</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D18" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E18" s="69" t="n"/>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="D55" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-19 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46159</v>
+        <v>46161</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="D23" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E23" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-22 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46161</v>
+        <v>46164</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="D55" s="68" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发3次，迟发1次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-23 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46164</v>
+        <v>46165</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="D31" s="71" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发3次</t>
+          <t>累计未发4次，迟发3次</t>
         </is>
       </c>
       <c r="E31" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-24 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46165</v>
+        <v>46166</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="D32" s="71" t="inlineStr">
         <is>
-          <t>累计未发5次，迟发3次</t>
+          <t>累计未发6次，迟发3次</t>
         </is>
       </c>
       <c r="E32" s="69" t="inlineStr">

</xml_diff>

<commit_message>
report: update 2026-05-25 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="D26" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E26" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-26 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46167</v>
+        <v>46168</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D18" s="68" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发4次</t>
         </is>
       </c>
       <c r="E18" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-28 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46168</v>
+        <v>46170</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="D30" s="71" t="inlineStr">
         <is>
-          <t>累计迟发2次</t>
+          <t>迟发3次</t>
         </is>
       </c>
       <c r="E30" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-29 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3587,7 +3587,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D25" s="71" t="n"/>
+      <c r="D25" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E25" s="69" t="n"/>
       <c r="F25" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-05-30 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="D6" s="68" t="inlineStr">
         <is>
-          <t>累计未发5次</t>
+          <t>累计未发6次</t>
         </is>
       </c>
       <c r="E6" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-05-31 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="D5" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E5" s="69" t="n"/>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D18" s="68" t="inlineStr">
         <is>
-          <t>累计未发4次</t>
+          <t>累计未发5次</t>
         </is>
       </c>
       <c r="E18" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-06-01 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="D13" s="70" t="inlineStr">
         <is>
-          <t>累计未发4次，迟发1次</t>
+          <t>累计未发4次，迟发2次</t>
         </is>
       </c>
       <c r="E13" s="70" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-06-13 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46177</v>
+        <v>46186</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3701,7 +3701,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D31" s="71" t="n"/>
+      <c r="D31" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E31" s="69" t="n"/>
       <c r="F31" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-06-15 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46186</v>
+        <v>46188</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3830,7 +3830,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D36" s="73" t="n"/>
+      <c r="D36" s="73" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E36" s="69" t="n"/>
       <c r="F36" s="63" t="inlineStr">
         <is>
@@ -4380,7 +4384,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D58" s="68" t="n"/>
+      <c r="D58" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E58" s="69" t="n"/>
       <c r="F58" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-06-17 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46188</v>
+        <v>46190</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4259,7 +4259,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D53" s="70" t="n"/>
+      <c r="D53" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E53" s="69" t="n"/>
       <c r="F53" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-06-19 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46190</v>
+        <v>46192</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2824,7 +2824,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D5" s="68" t="n"/>
+      <c r="D5" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E5" s="69" t="n"/>
       <c r="F5" s="63" t="inlineStr">
         <is>
@@ -2988,7 +2992,7 @@
       </c>
       <c r="D8" s="68" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>迟发2次</t>
         </is>
       </c>
       <c r="E8" s="69" t="n"/>
@@ -3076,7 +3080,7 @@
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>迟发2次</t>
         </is>
       </c>
       <c r="E10" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-06-20 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3578,7 +3578,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D26" s="68" t="n"/>
+      <c r="D26" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E26" s="69" t="n"/>
       <c r="F26" s="63" t="inlineStr">
         <is>
@@ -3605,7 +3609,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D27" s="71" t="n"/>
+      <c r="D27" s="71" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E27" s="69" t="n"/>
       <c r="F27" s="63" t="inlineStr">
         <is>
@@ -3836,7 +3844,7 @@
       </c>
       <c r="D36" s="73" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E36" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-06-21 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46193</v>
+        <v>46194</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2888,7 +2888,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D6" s="68" t="n"/>
+      <c r="D6" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E6" s="69" t="n"/>
       <c r="F6" s="63" t="inlineStr">
         <is>
@@ -4121,7 +4125,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D47" s="68" t="n"/>
+      <c r="D47" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E47" s="71" t="n"/>
       <c r="F47" s="63" t="inlineStr">
         <is>
@@ -4528,7 +4536,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D63" s="68" t="n"/>
+      <c r="D63" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E63" s="69" t="n"/>
       <c r="F63" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-06-25 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46194</v>
+        <v>46198</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="D19" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E19" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-06-27 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46198</v>
+        <v>46200</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3975,7 +3975,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D41" s="71" t="n"/>
+      <c r="D41" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E41" s="69" t="n"/>
       <c r="F41" s="63" t="inlineStr">
         <is>
@@ -4075,7 +4079,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D45" s="71" t="n"/>
+      <c r="D45" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E45" s="69" t="n"/>
       <c r="F45" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-06-28 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3900,7 +3900,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D38" s="70" t="n"/>
+      <c r="D38" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E38" s="69" t="n"/>
       <c r="F38" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-06-30 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46201</v>
+        <v>46203</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="D19" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E19" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-07-01 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46203</v>
+        <v>46204</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4191,7 +4191,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D49" s="71" t="n"/>
+      <c r="D49" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E49" s="69" t="n"/>
       <c r="F49" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-07-02 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46204</v>
+        <v>46205</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4033,7 +4033,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D43" s="68" t="n"/>
+      <c r="D43" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E43" s="69" t="n"/>
       <c r="F43" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-07-03 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="D6" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E6" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-07-04 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="D8" s="68" t="inlineStr">
         <is>
-          <t>迟发2次</t>
+          <t>迟发3次</t>
         </is>
       </c>
       <c r="E8" s="69" t="n"/>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>迟发2次</t>
+          <t>迟发3次</t>
         </is>
       </c>
       <c r="E10" s="69" t="n"/>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="D36" s="73" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E36" s="69" t="n"/>
@@ -4353,7 +4353,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D55" s="70" t="n"/>
+      <c r="D55" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E55" s="69" t="n"/>
       <c r="F55" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-07-05 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="D6" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E6" s="69" t="n"/>
@@ -3796,7 +3796,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D34" s="71" t="n"/>
+      <c r="D34" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E34" s="69" t="n"/>
       <c r="F34" s="63" t="inlineStr">
         <is>
@@ -3902,7 +3906,7 @@
       </c>
       <c r="D38" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E38" s="69" t="n"/>
@@ -4407,7 +4411,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D57" s="68" t="n"/>
+      <c r="D57" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E57" s="69" t="n"/>
       <c r="F57" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-07-06 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3692,7 +3692,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D30" s="68" t="n"/>
+      <c r="D30" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E30" s="69" t="n"/>
       <c r="F30" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-07-07 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="D8" s="68" t="inlineStr">
         <is>
-          <t>迟发3次</t>
+          <t>迟发4次</t>
         </is>
       </c>
       <c r="E8" s="69" t="n"/>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>迟发3次</t>
+          <t>迟发4次</t>
         </is>
       </c>
       <c r="E10" s="69" t="n"/>
@@ -3258,7 +3258,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D14" s="70" t="n"/>
+      <c r="D14" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E14" s="69" t="n"/>
       <c r="F14" s="63" t="inlineStr">
         <is>
@@ -3291,7 +3295,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D15" s="70" t="n"/>
+      <c r="D15" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E15" s="69" t="n"/>
       <c r="F15" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-07-18 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="27040" windowHeight="16400" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16400" windowWidth="27040" xWindow="0" yWindow="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026年日报'!$A$2:$F$61</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'2026年日报'!$A$2:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,257 +449,257 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1">
+    <xf applyAlignment="1" borderId="7" fillId="7" fontId="0" numFmtId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="83">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="3" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="5" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="5" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="10" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="11" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="12" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="16" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="14" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="9" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -1073,16 +1073,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1557,7 +1557,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1642,7 +1642,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D40" s="46" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D48" s="51" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -2619,26 +2619,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46215</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+        <v>46221</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>区域</t>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2808,7 +2808,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2872,7 +2872,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2927,7 +2927,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2978,7 +2978,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3024,7 +3024,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3066,7 +3066,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3112,7 +3112,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3158,7 +3158,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3200,7 +3200,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3242,7 +3242,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3279,7 +3279,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="15" s="78">
       <c r="A15" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3310,7 +3310,7 @@
       <c r="H15" s="23" t="n"/>
       <c r="J15" s="67" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3343,7 +3343,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="G17" s="67" t="n"/>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="G18" s="67" t="n"/>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G19" s="67" t="n"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3447,7 +3447,7 @@
       </c>
       <c r="G20" s="67" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="G21" s="67" t="n"/>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G22" s="67" t="n"/>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="G23" s="67" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="G24" s="67" t="n"/>
     </row>
-    <row r="25" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="25" s="78">
       <c r="A25" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3574,7 +3574,7 @@
       <c r="H25" s="67" t="n"/>
       <c r="J25" s="67" t="n"/>
     </row>
-    <row r="26" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="26" s="78">
       <c r="A26" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3605,7 +3605,7 @@
       <c r="H26" s="67" t="n"/>
       <c r="J26" s="67" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="G27" s="67" t="n"/>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="G28" s="67" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3684,7 +3684,7 @@
       </c>
       <c r="G29" s="67" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="D30" s="68" t="inlineStr">
         <is>
-          <t>迟发2次</t>
+          <t>迟发3次</t>
         </is>
       </c>
       <c r="E30" s="69" t="n"/>
@@ -3713,7 +3713,7 @@
       </c>
       <c r="G30" s="67" t="n"/>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="G31" s="67" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="G32" s="67" t="n"/>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="G33" s="67" t="n"/>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="D34" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E34" s="69" t="n"/>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="G34" s="67" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="G35" s="67" t="n"/>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="G36" s="67" t="n"/>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="G37" s="67" t="n"/>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="G38" s="67" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="G39" s="67" t="n"/>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="G40" s="67" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="G41" s="67" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="G42" s="67" t="n"/>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="G43" s="67" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="G44" s="67" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G45" s="67" t="n"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4145,7 +4145,7 @@
       </c>
       <c r="G46" s="67" t="n"/>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="G47" s="67" t="n"/>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="G48" s="67" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="G49" s="67" t="n"/>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="G50" s="67" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="G51" s="67" t="n"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="G52" s="67" t="n"/>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="72" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -4332,7 +4332,7 @@
       </c>
       <c r="G53" s="67" t="n"/>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="58" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -4357,7 +4357,7 @@
       </c>
       <c r="G54" s="67" t="n"/>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4386,7 +4386,7 @@
       </c>
       <c r="G55" s="67" t="n"/>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="G56" s="67" t="n"/>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="58" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="G57" s="67" t="n"/>
     </row>
-    <row r="58" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="58" s="53">
       <c r="A58" s="60" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="G58" s="67" t="n"/>
     </row>
-    <row r="59" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="59" s="53">
       <c r="A59" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="G59" s="67" t="n"/>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="60" s="53">
       <c r="A60" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="G60" s="67" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="61" s="53">
       <c r="A61" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="G61" s="67" t="n"/>
     </row>
-    <row r="62" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="62" s="53">
       <c r="A62" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4572,7 +4572,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="63" s="53">
       <c r="A63" s="60" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -4596,234 +4596,234 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1" s="53">
-      <c r="A64" t="inlineStr">
+    <row customHeight="1" ht="16" r="64" s="53">
+      <c r="A64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="0" t="inlineStr">
         <is>
           <t>合肥包河中心</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D64" s="0" t="inlineStr">
         <is>
           <t>累计未发1次</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1" s="53"/>
-    <row r="66" ht="16" customHeight="1" s="53"/>
-    <row r="67" ht="16" customHeight="1" s="53"/>
-    <row r="68" ht="16" customHeight="1" s="53"/>
-    <row r="69" ht="16" customHeight="1" s="53"/>
-    <row r="70" ht="16" customHeight="1" s="53"/>
-    <row r="71" ht="16" customHeight="1" s="53"/>
-    <row r="72" ht="16" customHeight="1" s="53"/>
-    <row r="73" ht="16" customHeight="1" s="53"/>
-    <row r="74" ht="16" customHeight="1" s="53"/>
-    <row r="75" ht="16" customHeight="1" s="53"/>
-    <row r="76" ht="16" customHeight="1" s="53"/>
-    <row r="77" ht="16" customHeight="1" s="53"/>
-    <row r="78" ht="16" customHeight="1" s="53"/>
-    <row r="79" ht="16" customHeight="1" s="53"/>
-    <row r="80" ht="16" customHeight="1" s="53"/>
-    <row r="81" ht="16" customHeight="1" s="53"/>
-    <row r="82" ht="16" customHeight="1" s="53"/>
-    <row r="83" ht="16" customHeight="1" s="53"/>
-    <row r="84" ht="16" customHeight="1" s="53"/>
-    <row r="85" ht="16" customHeight="1" s="53"/>
-    <row r="86" ht="16" customHeight="1" s="53"/>
-    <row r="87" ht="16" customHeight="1" s="53"/>
-    <row r="88" ht="16" customHeight="1" s="53"/>
-    <row r="89" ht="16" customHeight="1" s="53"/>
-    <row r="90" ht="16" customHeight="1" s="53"/>
-    <row r="91" ht="16" customHeight="1" s="53"/>
-    <row r="92" ht="16" customHeight="1" s="53"/>
-    <row r="93" ht="16" customHeight="1" s="53"/>
-    <row r="94" ht="16" customHeight="1" s="53"/>
-    <row r="95" ht="16" customHeight="1" s="53"/>
-    <row r="96" ht="16" customHeight="1" s="53"/>
-    <row r="97" ht="16" customHeight="1" s="53"/>
-    <row r="98" ht="16" customHeight="1" s="53"/>
-    <row r="99" ht="16" customHeight="1" s="53"/>
-    <row r="100" ht="16" customHeight="1" s="53"/>
-    <row r="101" ht="16" customHeight="1" s="53"/>
-    <row r="102" ht="16" customHeight="1" s="53"/>
-    <row r="103" ht="16" customHeight="1" s="53"/>
-    <row r="104" ht="16" customHeight="1" s="53"/>
-    <row r="105" ht="16" customHeight="1" s="53"/>
-    <row r="106" ht="16" customHeight="1" s="53"/>
-    <row r="107" ht="16" customHeight="1" s="53"/>
-    <row r="108" ht="16" customHeight="1" s="53"/>
-    <row r="109" ht="16" customHeight="1" s="53"/>
-    <row r="110" ht="16" customHeight="1" s="53"/>
-    <row r="111" ht="16" customHeight="1" s="53"/>
-    <row r="112" ht="16" customHeight="1" s="53"/>
-    <row r="113" ht="16" customHeight="1" s="53"/>
-    <row r="114" ht="16" customHeight="1" s="53"/>
-    <row r="115" ht="16" customHeight="1" s="53"/>
-    <row r="116" ht="16" customHeight="1" s="53"/>
-    <row r="117" ht="16" customHeight="1" s="53"/>
-    <row r="118" ht="16" customHeight="1" s="53"/>
-    <row r="119" ht="16" customHeight="1" s="53"/>
-    <row r="120" ht="16" customHeight="1" s="53"/>
-    <row r="121" ht="16" customHeight="1" s="53"/>
-    <row r="122" ht="16" customHeight="1" s="53"/>
-    <row r="123" ht="16" customHeight="1" s="53"/>
-    <row r="124" ht="16" customHeight="1" s="53"/>
-    <row r="125" ht="16" customHeight="1" s="53"/>
-    <row r="126" ht="16" customHeight="1" s="53"/>
-    <row r="127" ht="16" customHeight="1" s="53"/>
-    <row r="128" ht="16" customHeight="1" s="53"/>
-    <row r="129" ht="16" customHeight="1" s="53"/>
-    <row r="130" ht="16" customHeight="1" s="53"/>
-    <row r="131" ht="16" customHeight="1" s="53"/>
-    <row r="132" ht="16" customHeight="1" s="53"/>
-    <row r="133" ht="16" customHeight="1" s="53"/>
-    <row r="134" ht="16" customHeight="1" s="53"/>
-    <row r="135" ht="16" customHeight="1" s="53"/>
-    <row r="136" ht="16" customHeight="1" s="53"/>
-    <row r="137" ht="16" customHeight="1" s="53"/>
-    <row r="138" ht="16" customHeight="1" s="53"/>
-    <row r="139" ht="16" customHeight="1" s="53"/>
-    <row r="140" ht="16" customHeight="1" s="53"/>
-    <row r="141" ht="16" customHeight="1" s="53"/>
-    <row r="142" ht="16" customHeight="1" s="53"/>
-    <row r="143" ht="16" customHeight="1" s="53"/>
-    <row r="144" ht="16" customHeight="1" s="53"/>
-    <row r="145" ht="16" customHeight="1" s="53"/>
-    <row r="146" ht="16" customHeight="1" s="53"/>
-    <row r="147" ht="16" customHeight="1" s="53"/>
-    <row r="148" ht="16" customHeight="1" s="53"/>
-    <row r="149" ht="16" customHeight="1" s="53"/>
-    <row r="150" ht="16" customHeight="1" s="53"/>
-    <row r="151" ht="16" customHeight="1" s="53"/>
-    <row r="152" ht="16" customHeight="1" s="53"/>
-    <row r="153" ht="16" customHeight="1" s="53"/>
-    <row r="154" ht="16" customHeight="1" s="53"/>
-    <row r="155" ht="16" customHeight="1" s="53"/>
-    <row r="156" ht="16" customHeight="1" s="53"/>
-    <row r="157" ht="16" customHeight="1" s="53"/>
-    <row r="158" ht="16" customHeight="1" s="53"/>
-    <row r="159" ht="16" customHeight="1" s="53"/>
-    <row r="160" ht="16" customHeight="1" s="53"/>
-    <row r="161" ht="16" customHeight="1" s="53"/>
-    <row r="162" ht="16" customHeight="1" s="53"/>
-    <row r="163" ht="16" customHeight="1" s="53"/>
-    <row r="164" ht="16" customHeight="1" s="53"/>
-    <row r="165" ht="16" customHeight="1" s="53"/>
-    <row r="166" ht="16" customHeight="1" s="53"/>
-    <row r="167" ht="16" customHeight="1" s="53"/>
-    <row r="168" ht="16" customHeight="1" s="53"/>
-    <row r="169" ht="16" customHeight="1" s="53"/>
-    <row r="170" ht="16" customHeight="1" s="53"/>
-    <row r="171" ht="16" customHeight="1" s="53"/>
-    <row r="172" ht="16" customHeight="1" s="53"/>
-    <row r="173" ht="16" customHeight="1" s="53"/>
-    <row r="174" ht="16" customHeight="1" s="53"/>
-    <row r="175" ht="16" customHeight="1" s="53"/>
-    <row r="176" ht="16" customHeight="1" s="53"/>
-    <row r="177" ht="16" customHeight="1" s="53"/>
-    <row r="178" ht="16" customHeight="1" s="53"/>
-    <row r="179" ht="16" customHeight="1" s="53"/>
-    <row r="180" ht="16" customHeight="1" s="53"/>
-    <row r="181" ht="16" customHeight="1" s="53"/>
-    <row r="182" ht="16" customHeight="1" s="53"/>
-    <row r="183" ht="16" customHeight="1" s="53"/>
-    <row r="184" ht="16" customHeight="1" s="53"/>
-    <row r="185" ht="16" customHeight="1" s="53"/>
-    <row r="186" ht="16" customHeight="1" s="53"/>
-    <row r="187" ht="16" customHeight="1" s="53"/>
-    <row r="188" ht="16" customHeight="1" s="53"/>
-    <row r="189" ht="16" customHeight="1" s="53"/>
-    <row r="190" ht="16" customHeight="1" s="53"/>
-    <row r="191" ht="16" customHeight="1" s="53"/>
-    <row r="192" ht="16" customHeight="1" s="53"/>
-    <row r="193" ht="16" customHeight="1" s="53"/>
-    <row r="194" ht="16" customHeight="1" s="53"/>
-    <row r="195" ht="16" customHeight="1" s="53"/>
-    <row r="196" ht="16" customHeight="1" s="53"/>
-    <row r="197" ht="16" customHeight="1" s="53"/>
-    <row r="198" ht="16" customHeight="1" s="53"/>
-    <row r="199" ht="16" customHeight="1" s="53"/>
-    <row r="200" ht="16" customHeight="1" s="53"/>
-    <row r="201" ht="16" customHeight="1" s="53"/>
-    <row r="202" ht="16" customHeight="1" s="53"/>
-    <row r="203" ht="16" customHeight="1" s="53"/>
-    <row r="204" ht="16" customHeight="1" s="53"/>
-    <row r="205" ht="16" customHeight="1" s="53"/>
-    <row r="206" ht="16" customHeight="1" s="53"/>
-    <row r="207" ht="16" customHeight="1" s="53"/>
-    <row r="208" ht="16" customHeight="1" s="53"/>
-    <row r="209" ht="16" customHeight="1" s="53"/>
-    <row r="210" ht="16" customHeight="1" s="53"/>
-    <row r="211" ht="16" customHeight="1" s="53"/>
-    <row r="212" ht="16" customHeight="1" s="53"/>
-    <row r="213" ht="16" customHeight="1" s="53"/>
-    <row r="214" ht="16" customHeight="1" s="53"/>
-    <row r="215" ht="16" customHeight="1" s="53"/>
-    <row r="216" ht="16" customHeight="1" s="53"/>
-    <row r="217" ht="16" customHeight="1" s="53"/>
-    <row r="218" ht="16" customHeight="1" s="53"/>
-    <row r="219" ht="16" customHeight="1" s="53"/>
-    <row r="220" ht="16" customHeight="1" s="53"/>
-    <row r="221" ht="16" customHeight="1" s="53"/>
-    <row r="222" ht="16" customHeight="1" s="53"/>
-    <row r="223" ht="16" customHeight="1" s="53"/>
-    <row r="224" ht="16" customHeight="1" s="53"/>
-    <row r="225" ht="16" customHeight="1" s="53"/>
-    <row r="226" ht="16" customHeight="1" s="53"/>
-    <row r="227" ht="16" customHeight="1" s="53"/>
-    <row r="228" ht="16" customHeight="1" s="53"/>
-    <row r="229" ht="16" customHeight="1" s="53"/>
-    <row r="230" ht="16" customHeight="1" s="53"/>
-    <row r="231" ht="16" customHeight="1" s="53"/>
-    <row r="232" ht="16" customHeight="1" s="53"/>
-    <row r="233" ht="16" customHeight="1" s="53"/>
-    <row r="234" ht="16" customHeight="1" s="53"/>
-    <row r="235" ht="16" customHeight="1" s="53"/>
-    <row r="236" ht="16" customHeight="1" s="53"/>
-    <row r="237" ht="16" customHeight="1" s="53"/>
-    <row r="238" ht="16" customHeight="1" s="53"/>
-    <row r="239" ht="16" customHeight="1" s="53"/>
-    <row r="240" ht="16" customHeight="1" s="53"/>
-    <row r="241" ht="16" customHeight="1" s="53"/>
-    <row r="242" ht="16" customHeight="1" s="53"/>
-    <row r="243" ht="16" customHeight="1" s="53"/>
-    <row r="244" ht="16" customHeight="1" s="53"/>
-    <row r="245" ht="16" customHeight="1" s="53"/>
-    <row r="246" ht="16" customHeight="1" s="53"/>
-    <row r="247" ht="16" customHeight="1" s="53"/>
-    <row r="248" ht="16" customHeight="1" s="53"/>
-    <row r="249" ht="16" customHeight="1" s="53"/>
-    <row r="250" ht="16" customHeight="1" s="53"/>
-    <row r="251" ht="16" customHeight="1" s="53"/>
-    <row r="252" ht="16" customHeight="1" s="53"/>
-    <row r="253" ht="16" customHeight="1" s="53"/>
-    <row r="254" ht="16" customHeight="1" s="53"/>
-    <row r="255" ht="16" customHeight="1" s="53"/>
-    <row r="256" ht="16" customHeight="1" s="53"/>
-    <row r="257" ht="16" customHeight="1" s="53"/>
-    <row r="258" ht="16" customHeight="1" s="53"/>
-    <row r="259" ht="16" customHeight="1" s="53"/>
-    <row r="260" ht="16" customHeight="1" s="53"/>
-    <row r="261" ht="16" customHeight="1" s="53"/>
-    <row r="262" ht="16" customHeight="1" s="53"/>
+    <row customHeight="1" ht="16" r="65" s="53"/>
+    <row customHeight="1" ht="16" r="66" s="53"/>
+    <row customHeight="1" ht="16" r="67" s="53"/>
+    <row customHeight="1" ht="16" r="68" s="53"/>
+    <row customHeight="1" ht="16" r="69" s="53"/>
+    <row customHeight="1" ht="16" r="70" s="53"/>
+    <row customHeight="1" ht="16" r="71" s="53"/>
+    <row customHeight="1" ht="16" r="72" s="53"/>
+    <row customHeight="1" ht="16" r="73" s="53"/>
+    <row customHeight="1" ht="16" r="74" s="53"/>
+    <row customHeight="1" ht="16" r="75" s="53"/>
+    <row customHeight="1" ht="16" r="76" s="53"/>
+    <row customHeight="1" ht="16" r="77" s="53"/>
+    <row customHeight="1" ht="16" r="78" s="53"/>
+    <row customHeight="1" ht="16" r="79" s="53"/>
+    <row customHeight="1" ht="16" r="80" s="53"/>
+    <row customHeight="1" ht="16" r="81" s="53"/>
+    <row customHeight="1" ht="16" r="82" s="53"/>
+    <row customHeight="1" ht="16" r="83" s="53"/>
+    <row customHeight="1" ht="16" r="84" s="53"/>
+    <row customHeight="1" ht="16" r="85" s="53"/>
+    <row customHeight="1" ht="16" r="86" s="53"/>
+    <row customHeight="1" ht="16" r="87" s="53"/>
+    <row customHeight="1" ht="16" r="88" s="53"/>
+    <row customHeight="1" ht="16" r="89" s="53"/>
+    <row customHeight="1" ht="16" r="90" s="53"/>
+    <row customHeight="1" ht="16" r="91" s="53"/>
+    <row customHeight="1" ht="16" r="92" s="53"/>
+    <row customHeight="1" ht="16" r="93" s="53"/>
+    <row customHeight="1" ht="16" r="94" s="53"/>
+    <row customHeight="1" ht="16" r="95" s="53"/>
+    <row customHeight="1" ht="16" r="96" s="53"/>
+    <row customHeight="1" ht="16" r="97" s="53"/>
+    <row customHeight="1" ht="16" r="98" s="53"/>
+    <row customHeight="1" ht="16" r="99" s="53"/>
+    <row customHeight="1" ht="16" r="100" s="53"/>
+    <row customHeight="1" ht="16" r="101" s="53"/>
+    <row customHeight="1" ht="16" r="102" s="53"/>
+    <row customHeight="1" ht="16" r="103" s="53"/>
+    <row customHeight="1" ht="16" r="104" s="53"/>
+    <row customHeight="1" ht="16" r="105" s="53"/>
+    <row customHeight="1" ht="16" r="106" s="53"/>
+    <row customHeight="1" ht="16" r="107" s="53"/>
+    <row customHeight="1" ht="16" r="108" s="53"/>
+    <row customHeight="1" ht="16" r="109" s="53"/>
+    <row customHeight="1" ht="16" r="110" s="53"/>
+    <row customHeight="1" ht="16" r="111" s="53"/>
+    <row customHeight="1" ht="16" r="112" s="53"/>
+    <row customHeight="1" ht="16" r="113" s="53"/>
+    <row customHeight="1" ht="16" r="114" s="53"/>
+    <row customHeight="1" ht="16" r="115" s="53"/>
+    <row customHeight="1" ht="16" r="116" s="53"/>
+    <row customHeight="1" ht="16" r="117" s="53"/>
+    <row customHeight="1" ht="16" r="118" s="53"/>
+    <row customHeight="1" ht="16" r="119" s="53"/>
+    <row customHeight="1" ht="16" r="120" s="53"/>
+    <row customHeight="1" ht="16" r="121" s="53"/>
+    <row customHeight="1" ht="16" r="122" s="53"/>
+    <row customHeight="1" ht="16" r="123" s="53"/>
+    <row customHeight="1" ht="16" r="124" s="53"/>
+    <row customHeight="1" ht="16" r="125" s="53"/>
+    <row customHeight="1" ht="16" r="126" s="53"/>
+    <row customHeight="1" ht="16" r="127" s="53"/>
+    <row customHeight="1" ht="16" r="128" s="53"/>
+    <row customHeight="1" ht="16" r="129" s="53"/>
+    <row customHeight="1" ht="16" r="130" s="53"/>
+    <row customHeight="1" ht="16" r="131" s="53"/>
+    <row customHeight="1" ht="16" r="132" s="53"/>
+    <row customHeight="1" ht="16" r="133" s="53"/>
+    <row customHeight="1" ht="16" r="134" s="53"/>
+    <row customHeight="1" ht="16" r="135" s="53"/>
+    <row customHeight="1" ht="16" r="136" s="53"/>
+    <row customHeight="1" ht="16" r="137" s="53"/>
+    <row customHeight="1" ht="16" r="138" s="53"/>
+    <row customHeight="1" ht="16" r="139" s="53"/>
+    <row customHeight="1" ht="16" r="140" s="53"/>
+    <row customHeight="1" ht="16" r="141" s="53"/>
+    <row customHeight="1" ht="16" r="142" s="53"/>
+    <row customHeight="1" ht="16" r="143" s="53"/>
+    <row customHeight="1" ht="16" r="144" s="53"/>
+    <row customHeight="1" ht="16" r="145" s="53"/>
+    <row customHeight="1" ht="16" r="146" s="53"/>
+    <row customHeight="1" ht="16" r="147" s="53"/>
+    <row customHeight="1" ht="16" r="148" s="53"/>
+    <row customHeight="1" ht="16" r="149" s="53"/>
+    <row customHeight="1" ht="16" r="150" s="53"/>
+    <row customHeight="1" ht="16" r="151" s="53"/>
+    <row customHeight="1" ht="16" r="152" s="53"/>
+    <row customHeight="1" ht="16" r="153" s="53"/>
+    <row customHeight="1" ht="16" r="154" s="53"/>
+    <row customHeight="1" ht="16" r="155" s="53"/>
+    <row customHeight="1" ht="16" r="156" s="53"/>
+    <row customHeight="1" ht="16" r="157" s="53"/>
+    <row customHeight="1" ht="16" r="158" s="53"/>
+    <row customHeight="1" ht="16" r="159" s="53"/>
+    <row customHeight="1" ht="16" r="160" s="53"/>
+    <row customHeight="1" ht="16" r="161" s="53"/>
+    <row customHeight="1" ht="16" r="162" s="53"/>
+    <row customHeight="1" ht="16" r="163" s="53"/>
+    <row customHeight="1" ht="16" r="164" s="53"/>
+    <row customHeight="1" ht="16" r="165" s="53"/>
+    <row customHeight="1" ht="16" r="166" s="53"/>
+    <row customHeight="1" ht="16" r="167" s="53"/>
+    <row customHeight="1" ht="16" r="168" s="53"/>
+    <row customHeight="1" ht="16" r="169" s="53"/>
+    <row customHeight="1" ht="16" r="170" s="53"/>
+    <row customHeight="1" ht="16" r="171" s="53"/>
+    <row customHeight="1" ht="16" r="172" s="53"/>
+    <row customHeight="1" ht="16" r="173" s="53"/>
+    <row customHeight="1" ht="16" r="174" s="53"/>
+    <row customHeight="1" ht="16" r="175" s="53"/>
+    <row customHeight="1" ht="16" r="176" s="53"/>
+    <row customHeight="1" ht="16" r="177" s="53"/>
+    <row customHeight="1" ht="16" r="178" s="53"/>
+    <row customHeight="1" ht="16" r="179" s="53"/>
+    <row customHeight="1" ht="16" r="180" s="53"/>
+    <row customHeight="1" ht="16" r="181" s="53"/>
+    <row customHeight="1" ht="16" r="182" s="53"/>
+    <row customHeight="1" ht="16" r="183" s="53"/>
+    <row customHeight="1" ht="16" r="184" s="53"/>
+    <row customHeight="1" ht="16" r="185" s="53"/>
+    <row customHeight="1" ht="16" r="186" s="53"/>
+    <row customHeight="1" ht="16" r="187" s="53"/>
+    <row customHeight="1" ht="16" r="188" s="53"/>
+    <row customHeight="1" ht="16" r="189" s="53"/>
+    <row customHeight="1" ht="16" r="190" s="53"/>
+    <row customHeight="1" ht="16" r="191" s="53"/>
+    <row customHeight="1" ht="16" r="192" s="53"/>
+    <row customHeight="1" ht="16" r="193" s="53"/>
+    <row customHeight="1" ht="16" r="194" s="53"/>
+    <row customHeight="1" ht="16" r="195" s="53"/>
+    <row customHeight="1" ht="16" r="196" s="53"/>
+    <row customHeight="1" ht="16" r="197" s="53"/>
+    <row customHeight="1" ht="16" r="198" s="53"/>
+    <row customHeight="1" ht="16" r="199" s="53"/>
+    <row customHeight="1" ht="16" r="200" s="53"/>
+    <row customHeight="1" ht="16" r="201" s="53"/>
+    <row customHeight="1" ht="16" r="202" s="53"/>
+    <row customHeight="1" ht="16" r="203" s="53"/>
+    <row customHeight="1" ht="16" r="204" s="53"/>
+    <row customHeight="1" ht="16" r="205" s="53"/>
+    <row customHeight="1" ht="16" r="206" s="53"/>
+    <row customHeight="1" ht="16" r="207" s="53"/>
+    <row customHeight="1" ht="16" r="208" s="53"/>
+    <row customHeight="1" ht="16" r="209" s="53"/>
+    <row customHeight="1" ht="16" r="210" s="53"/>
+    <row customHeight="1" ht="16" r="211" s="53"/>
+    <row customHeight="1" ht="16" r="212" s="53"/>
+    <row customHeight="1" ht="16" r="213" s="53"/>
+    <row customHeight="1" ht="16" r="214" s="53"/>
+    <row customHeight="1" ht="16" r="215" s="53"/>
+    <row customHeight="1" ht="16" r="216" s="53"/>
+    <row customHeight="1" ht="16" r="217" s="53"/>
+    <row customHeight="1" ht="16" r="218" s="53"/>
+    <row customHeight="1" ht="16" r="219" s="53"/>
+    <row customHeight="1" ht="16" r="220" s="53"/>
+    <row customHeight="1" ht="16" r="221" s="53"/>
+    <row customHeight="1" ht="16" r="222" s="53"/>
+    <row customHeight="1" ht="16" r="223" s="53"/>
+    <row customHeight="1" ht="16" r="224" s="53"/>
+    <row customHeight="1" ht="16" r="225" s="53"/>
+    <row customHeight="1" ht="16" r="226" s="53"/>
+    <row customHeight="1" ht="16" r="227" s="53"/>
+    <row customHeight="1" ht="16" r="228" s="53"/>
+    <row customHeight="1" ht="16" r="229" s="53"/>
+    <row customHeight="1" ht="16" r="230" s="53"/>
+    <row customHeight="1" ht="16" r="231" s="53"/>
+    <row customHeight="1" ht="16" r="232" s="53"/>
+    <row customHeight="1" ht="16" r="233" s="53"/>
+    <row customHeight="1" ht="16" r="234" s="53"/>
+    <row customHeight="1" ht="16" r="235" s="53"/>
+    <row customHeight="1" ht="16" r="236" s="53"/>
+    <row customHeight="1" ht="16" r="237" s="53"/>
+    <row customHeight="1" ht="16" r="238" s="53"/>
+    <row customHeight="1" ht="16" r="239" s="53"/>
+    <row customHeight="1" ht="16" r="240" s="53"/>
+    <row customHeight="1" ht="16" r="241" s="53"/>
+    <row customHeight="1" ht="16" r="242" s="53"/>
+    <row customHeight="1" ht="16" r="243" s="53"/>
+    <row customHeight="1" ht="16" r="244" s="53"/>
+    <row customHeight="1" ht="16" r="245" s="53"/>
+    <row customHeight="1" ht="16" r="246" s="53"/>
+    <row customHeight="1" ht="16" r="247" s="53"/>
+    <row customHeight="1" ht="16" r="248" s="53"/>
+    <row customHeight="1" ht="16" r="249" s="53"/>
+    <row customHeight="1" ht="16" r="250" s="53"/>
+    <row customHeight="1" ht="16" r="251" s="53"/>
+    <row customHeight="1" ht="16" r="252" s="53"/>
+    <row customHeight="1" ht="16" r="253" s="53"/>
+    <row customHeight="1" ht="16" r="254" s="53"/>
+    <row customHeight="1" ht="16" r="255" s="53"/>
+    <row customHeight="1" ht="16" r="256" s="53"/>
+    <row customHeight="1" ht="16" r="257" s="53"/>
+    <row customHeight="1" ht="16" r="258" s="53"/>
+    <row customHeight="1" ht="16" r="259" s="53"/>
+    <row customHeight="1" ht="16" r="260" s="53"/>
+    <row customHeight="1" ht="16" r="261" s="53"/>
+    <row customHeight="1" ht="16" r="262" s="53"/>
   </sheetData>
   <autoFilter ref="A2:F61"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -4836,17 +4836,17 @@
   <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -4869,7 +4869,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>区域</t>
@@ -4955,7 +4955,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -4998,7 +4998,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5080,7 +5080,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5125,7 +5125,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5164,7 +5164,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5201,7 +5201,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5230,7 +5230,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5269,7 +5269,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5306,7 +5306,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5343,7 +5343,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5382,7 +5382,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5419,7 +5419,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5446,7 +5446,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="10" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5474,7 +5474,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5502,7 +5502,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5530,7 +5530,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5560,7 +5560,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5590,7 +5590,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5654,7 +5654,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5684,7 +5684,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5722,7 +5722,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5752,7 +5752,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5784,7 +5784,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5818,7 +5818,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5850,7 +5850,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5878,7 +5878,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5914,7 +5914,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5941,7 +5941,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="10" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5973,7 +5973,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6005,7 +6005,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6030,7 +6030,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6060,7 +6060,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6090,7 +6090,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6124,7 +6124,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6154,7 +6154,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6182,7 +6182,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6210,7 +6210,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6238,7 +6238,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6266,7 +6266,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6294,7 +6294,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6322,7 +6322,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6350,7 +6350,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6378,7 +6378,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6416,7 +6416,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6446,7 +6446,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6482,7 +6482,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6516,7 +6516,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6552,7 +6552,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6584,7 +6584,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -7232,7 +7232,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -7245,17 +7245,17 @@
   <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -7278,7 +7278,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>区域</t>
@@ -7364,7 +7364,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7410,7 +7410,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7447,7 +7447,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7493,7 +7493,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7539,7 +7539,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7587,7 +7587,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7624,7 +7624,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7661,7 +7661,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7709,7 +7709,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7755,7 +7755,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7792,7 +7792,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7829,7 +7829,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7875,7 +7875,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7903,7 +7903,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -7931,7 +7931,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -7959,7 +7959,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -7987,7 +7987,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8015,7 +8015,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8043,7 +8043,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8071,7 +8071,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8099,7 +8099,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8127,7 +8127,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8155,7 +8155,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8183,7 +8183,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8211,7 +8211,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8239,7 +8239,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8269,7 +8269,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8297,7 +8297,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8325,7 +8325,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8353,7 +8353,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8381,7 +8381,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8437,7 +8437,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8467,7 +8467,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8495,7 +8495,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8523,7 +8523,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8551,7 +8551,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8579,7 +8579,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8609,7 +8609,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8641,7 +8641,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8669,7 +8669,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8697,7 +8697,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8725,7 +8725,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8753,7 +8753,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8781,7 +8781,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8813,7 +8813,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8845,7 +8845,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9521,7 +9521,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -9532,16 +9532,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
@@ -9551,7 +9551,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -9596,7 +9596,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9642,7 +9642,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9687,7 +9687,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9736,7 +9736,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9785,7 +9785,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9827,7 +9827,7 @@
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="35" t="n"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9862,7 +9862,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9902,7 +9902,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9938,7 +9938,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -9974,7 +9974,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10010,7 +10010,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10051,7 +10051,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10082,7 +10082,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10104,7 +10104,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10121,7 +10121,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10138,7 +10138,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10160,7 +10160,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10177,7 +10177,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10195,7 +10195,7 @@
       </c>
       <c r="D20" s="39" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10217,7 +10217,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10239,7 +10239,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10261,7 +10261,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10283,7 +10283,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10301,7 +10301,7 @@
       </c>
       <c r="D25" s="36" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10323,7 +10323,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10345,7 +10345,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10367,7 +10367,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10389,7 +10389,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10411,7 +10411,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10433,7 +10433,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10460,7 +10460,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10482,7 +10482,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10504,7 +10504,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10526,7 +10526,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10570,7 +10570,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10592,7 +10592,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10609,7 +10609,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10631,7 +10631,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10649,7 +10649,7 @@
       </c>
       <c r="D41" s="46" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10671,7 +10671,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10689,7 +10689,7 @@
       </c>
       <c r="D43" s="46" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10707,7 +10707,7 @@
       </c>
       <c r="E44" s="46" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10729,7 +10729,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10751,7 +10751,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10773,7 +10773,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10795,7 +10795,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10817,7 +10817,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10840,7 +10840,7 @@
       </c>
       <c r="E50" s="49" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10862,7 +10862,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10906,7 +10906,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="55" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -10928,7 +10928,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="55" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10972,7 +10972,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10990,7 +10990,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -11001,18 +11001,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6.83203125" customWidth="1" style="23" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="23" min="2" max="2"/>
-    <col width="19.6640625" customWidth="1" style="23" min="3" max="3"/>
-    <col width="13" customWidth="1" style="23" min="4" max="4"/>
-    <col hidden="1" width="30.5" customWidth="1" style="23" min="5" max="6"/>
-    <col width="30.5" customWidth="1" style="23" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="23" min="8" max="26"/>
+    <col customWidth="1" max="1" min="1" style="23" width="6.83203125"/>
+    <col customWidth="1" max="2" min="2" style="23" width="8.83203125"/>
+    <col customWidth="1" max="3" min="3" style="23" width="19.6640625"/>
+    <col customWidth="1" max="4" min="4" style="23" width="13"/>
+    <col customWidth="1" hidden="1" max="6" min="5" style="23" width="30.5"/>
+    <col customWidth="1" max="7" min="7" style="23" width="30.5"/>
+    <col customWidth="1" max="26" min="8" style="23" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="1" s="53">
       <c r="A1" s="21" t="n"/>
       <c r="B1" s="22" t="inlineStr">
         <is>
@@ -11054,7 +11054,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="2" s="53">
       <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
@@ -11097,7 +11097,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="3" s="53">
       <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
@@ -11130,7 +11130,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="4" s="53">
       <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
@@ -11168,7 +11168,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="5" s="53">
       <c r="A5" s="24" t="n">
         <v>4</v>
       </c>
@@ -11211,7 +11211,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="6" s="53">
       <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
@@ -11244,7 +11244,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="7" s="53">
       <c r="A7" s="24" t="n">
         <v>6</v>
       </c>
@@ -11273,7 +11273,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="8" s="53">
       <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
@@ -11303,7 +11303,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="9" s="53">
       <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
@@ -11328,7 +11328,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="10" s="53">
       <c r="A10" s="24" t="n">
         <v>1</v>
       </c>
@@ -11353,7 +11353,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="11" s="53">
       <c r="A11" s="24" t="n">
         <v>2</v>
       </c>
@@ -11383,7 +11383,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="12" s="53">
       <c r="A12" s="24" t="n">
         <v>3</v>
       </c>
@@ -11408,7 +11408,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="13" s="53">
       <c r="A13" s="24" t="n">
         <v>4</v>
       </c>
@@ -11438,7 +11438,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="14" s="53">
       <c r="A14" s="24" t="n">
         <v>5</v>
       </c>
@@ -11458,7 +11458,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="15" s="53">
       <c r="A15" s="24" t="n">
         <v>6</v>
       </c>
@@ -11488,7 +11488,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="16" s="53">
       <c r="A16" s="24" t="n">
         <v>1</v>
       </c>
@@ -11513,7 +11513,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="17" s="53">
       <c r="A17" s="24" t="n">
         <v>2</v>
       </c>
@@ -11548,7 +11548,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="18" s="53">
       <c r="A18" s="24" t="n">
         <v>3</v>
       </c>
@@ -11583,7 +11583,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="19" s="53">
       <c r="A19" s="24" t="n">
         <v>4</v>
       </c>
@@ -11608,7 +11608,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="20" s="53">
       <c r="A20" s="24" t="n">
         <v>5</v>
       </c>
@@ -11638,7 +11638,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="21" s="53">
       <c r="A21" s="24" t="n">
         <v>6</v>
       </c>
@@ -11668,7 +11668,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="22" s="53">
       <c r="A22" s="24" t="n">
         <v>7</v>
       </c>
@@ -11698,7 +11698,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="23" s="53">
       <c r="A23" s="24" t="n">
         <v>8</v>
       </c>
@@ -11728,7 +11728,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="24" s="53">
       <c r="A24" s="24" t="n">
         <v>1</v>
       </c>
@@ -11758,7 +11758,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="25" s="53">
       <c r="A25" s="24" t="n">
         <v>2</v>
       </c>
@@ -11788,7 +11788,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="26" s="53">
       <c r="A26" s="24" t="n">
         <v>3</v>
       </c>
@@ -11813,7 +11813,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="27" s="53">
       <c r="A27" s="24" t="n">
         <v>4</v>
       </c>
@@ -11843,7 +11843,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="28" s="53">
       <c r="A28" s="24" t="n">
         <v>5</v>
       </c>
@@ -11873,7 +11873,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="29" s="53">
       <c r="A29" s="24" t="n">
         <v>6</v>
       </c>
@@ -11903,7 +11903,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="30" s="53">
       <c r="A30" s="24" t="n">
         <v>7</v>
       </c>
@@ -11938,7 +11938,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="31" s="53">
       <c r="A31" s="24" t="n">
         <v>8</v>
       </c>
@@ -11968,7 +11968,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="32" s="53">
       <c r="A32" s="24" t="n">
         <v>1</v>
       </c>
@@ -11998,7 +11998,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="33" s="53">
       <c r="A33" s="24" t="n">
         <v>2</v>
       </c>
@@ -12028,7 +12028,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="34" s="53">
       <c r="A34" s="24" t="n">
         <v>3</v>
       </c>
@@ -12058,7 +12058,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="35" s="53">
       <c r="A35" s="24" t="n">
         <v>4</v>
       </c>
@@ -12088,7 +12088,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="36" s="53">
       <c r="A36" s="24" t="n">
         <v>1</v>
       </c>
@@ -12118,7 +12118,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="37" s="53">
       <c r="A37" s="24" t="n">
         <v>2</v>
       </c>
@@ -12153,7 +12153,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="38" s="53">
       <c r="A38" s="24" t="n">
         <v>3</v>
       </c>
@@ -12184,6 +12184,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
report: update 2026-07-19 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="D5" s="68" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E5" s="69" t="n"/>
@@ -3945,7 +3945,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D39" s="70" t="n"/>
+      <c r="D39" s="70" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E39" s="69" t="n"/>
       <c r="F39" s="63" t="inlineStr">
         <is>
@@ -4055,7 +4059,7 @@
       </c>
       <c r="D43" s="68" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>迟发2次</t>
         </is>
       </c>
       <c r="E43" s="69" t="n"/>
@@ -4429,7 +4433,7 @@
       </c>
       <c r="D57" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E57" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-07-26 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="27040" windowHeight="16400" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16400" windowWidth="27040" xWindow="0" yWindow="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026年日报'!$A$2:$F$61</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'2026年日报'!$A$2:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,257 +449,257 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1">
+    <xf applyAlignment="1" borderId="7" fillId="7" fontId="0" numFmtId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="83">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="3" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="5" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="5" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="10" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="11" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="12" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="16" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="14" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="9" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -1073,16 +1073,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1557,7 +1557,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1642,7 +1642,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D40" s="46" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D48" s="51" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -2619,26 +2619,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46222</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+        <v>46229</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>区域</t>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2808,7 +2808,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2872,7 +2872,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2927,7 +2927,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2978,7 +2978,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3024,7 +3024,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3066,7 +3066,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3112,7 +3112,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3158,7 +3158,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3200,7 +3200,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3242,7 +3242,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3279,7 +3279,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="15" s="78">
       <c r="A15" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3310,7 +3310,7 @@
       <c r="H15" s="23" t="n"/>
       <c r="J15" s="67" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3343,7 +3343,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="G17" s="67" t="n"/>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="G18" s="67" t="n"/>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G19" s="67" t="n"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3447,7 +3447,7 @@
       </c>
       <c r="G20" s="67" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="G21" s="67" t="n"/>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G22" s="67" t="n"/>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="G23" s="67" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="G24" s="67" t="n"/>
     </row>
-    <row r="25" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="25" s="78">
       <c r="A25" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3574,7 +3574,7 @@
       <c r="H25" s="67" t="n"/>
       <c r="J25" s="67" t="n"/>
     </row>
-    <row r="26" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="26" s="78">
       <c r="A26" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3605,7 +3605,7 @@
       <c r="H26" s="67" t="n"/>
       <c r="J26" s="67" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="G27" s="67" t="n"/>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="G28" s="67" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3684,7 +3684,7 @@
       </c>
       <c r="G29" s="67" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3713,7 +3713,7 @@
       </c>
       <c r="G30" s="67" t="n"/>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="G31" s="67" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="G32" s="67" t="n"/>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="G33" s="67" t="n"/>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="G34" s="67" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="G35" s="67" t="n"/>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="G36" s="67" t="n"/>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="G37" s="67" t="n"/>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="G38" s="67" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="G39" s="67" t="n"/>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="G40" s="67" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G41" s="67" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="G42" s="67" t="n"/>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4070,7 +4070,7 @@
       </c>
       <c r="G43" s="67" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4095,7 +4095,7 @@
       </c>
       <c r="G44" s="67" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="G45" s="67" t="n"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4149,7 +4149,7 @@
       </c>
       <c r="G46" s="67" t="n"/>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="G47" s="67" t="n"/>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="G48" s="67" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="G49" s="67" t="n"/>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="G50" s="67" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="G51" s="67" t="n"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4307,7 +4307,7 @@
       </c>
       <c r="G52" s="67" t="n"/>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="72" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="D53" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E53" s="69" t="n"/>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="G53" s="67" t="n"/>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="58" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -4352,7 +4352,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D54" s="70" t="n"/>
+      <c r="D54" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E54" s="69" t="n"/>
       <c r="F54" s="63" t="inlineStr">
         <is>
@@ -4361,7 +4365,7 @@
       </c>
       <c r="G54" s="67" t="n"/>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4390,7 +4394,7 @@
       </c>
       <c r="G55" s="67" t="n"/>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4415,7 +4419,7 @@
       </c>
       <c r="G56" s="67" t="n"/>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="58" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4444,7 +4448,7 @@
       </c>
       <c r="G57" s="67" t="n"/>
     </row>
-    <row r="58" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="58" s="53">
       <c r="A58" s="60" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4460,7 +4464,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D58" s="68" t="n"/>
+      <c r="D58" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E58" s="69" t="n"/>
       <c r="F58" s="63" t="inlineStr">
         <is>
@@ -4469,7 +4477,7 @@
       </c>
       <c r="G58" s="67" t="n"/>
     </row>
-    <row r="59" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="59" s="53">
       <c r="A59" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4498,7 +4506,7 @@
       </c>
       <c r="G59" s="67" t="n"/>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="60" s="53">
       <c r="A60" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4523,7 +4531,7 @@
       </c>
       <c r="G60" s="67" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="61" s="53">
       <c r="A61" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4552,7 +4560,7 @@
       </c>
       <c r="G61" s="67" t="n"/>
     </row>
-    <row r="62" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="62" s="53">
       <c r="A62" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4576,7 +4584,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="63" s="53">
       <c r="A63" s="60" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -4592,7 +4600,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D63" s="68" t="n"/>
+      <c r="D63" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E63" s="69" t="n"/>
       <c r="F63" s="63" t="inlineStr">
         <is>
@@ -4600,7 +4612,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="64" s="53">
       <c r="A64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4627,207 +4639,207 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1" s="53"/>
-    <row r="66" ht="16" customHeight="1" s="53"/>
-    <row r="67" ht="16" customHeight="1" s="53"/>
-    <row r="68" ht="16" customHeight="1" s="53"/>
-    <row r="69" ht="16" customHeight="1" s="53"/>
-    <row r="70" ht="16" customHeight="1" s="53"/>
-    <row r="71" ht="16" customHeight="1" s="53"/>
-    <row r="72" ht="16" customHeight="1" s="53"/>
-    <row r="73" ht="16" customHeight="1" s="53"/>
-    <row r="74" ht="16" customHeight="1" s="53"/>
-    <row r="75" ht="16" customHeight="1" s="53"/>
-    <row r="76" ht="16" customHeight="1" s="53"/>
-    <row r="77" ht="16" customHeight="1" s="53"/>
-    <row r="78" ht="16" customHeight="1" s="53"/>
-    <row r="79" ht="16" customHeight="1" s="53"/>
-    <row r="80" ht="16" customHeight="1" s="53"/>
-    <row r="81" ht="16" customHeight="1" s="53"/>
-    <row r="82" ht="16" customHeight="1" s="53"/>
-    <row r="83" ht="16" customHeight="1" s="53"/>
-    <row r="84" ht="16" customHeight="1" s="53"/>
-    <row r="85" ht="16" customHeight="1" s="53"/>
-    <row r="86" ht="16" customHeight="1" s="53"/>
-    <row r="87" ht="16" customHeight="1" s="53"/>
-    <row r="88" ht="16" customHeight="1" s="53"/>
-    <row r="89" ht="16" customHeight="1" s="53"/>
-    <row r="90" ht="16" customHeight="1" s="53"/>
-    <row r="91" ht="16" customHeight="1" s="53"/>
-    <row r="92" ht="16" customHeight="1" s="53"/>
-    <row r="93" ht="16" customHeight="1" s="53"/>
-    <row r="94" ht="16" customHeight="1" s="53"/>
-    <row r="95" ht="16" customHeight="1" s="53"/>
-    <row r="96" ht="16" customHeight="1" s="53"/>
-    <row r="97" ht="16" customHeight="1" s="53"/>
-    <row r="98" ht="16" customHeight="1" s="53"/>
-    <row r="99" ht="16" customHeight="1" s="53"/>
-    <row r="100" ht="16" customHeight="1" s="53"/>
-    <row r="101" ht="16" customHeight="1" s="53"/>
-    <row r="102" ht="16" customHeight="1" s="53"/>
-    <row r="103" ht="16" customHeight="1" s="53"/>
-    <row r="104" ht="16" customHeight="1" s="53"/>
-    <row r="105" ht="16" customHeight="1" s="53"/>
-    <row r="106" ht="16" customHeight="1" s="53"/>
-    <row r="107" ht="16" customHeight="1" s="53"/>
-    <row r="108" ht="16" customHeight="1" s="53"/>
-    <row r="109" ht="16" customHeight="1" s="53"/>
-    <row r="110" ht="16" customHeight="1" s="53"/>
-    <row r="111" ht="16" customHeight="1" s="53"/>
-    <row r="112" ht="16" customHeight="1" s="53"/>
-    <row r="113" ht="16" customHeight="1" s="53"/>
-    <row r="114" ht="16" customHeight="1" s="53"/>
-    <row r="115" ht="16" customHeight="1" s="53"/>
-    <row r="116" ht="16" customHeight="1" s="53"/>
-    <row r="117" ht="16" customHeight="1" s="53"/>
-    <row r="118" ht="16" customHeight="1" s="53"/>
-    <row r="119" ht="16" customHeight="1" s="53"/>
-    <row r="120" ht="16" customHeight="1" s="53"/>
-    <row r="121" ht="16" customHeight="1" s="53"/>
-    <row r="122" ht="16" customHeight="1" s="53"/>
-    <row r="123" ht="16" customHeight="1" s="53"/>
-    <row r="124" ht="16" customHeight="1" s="53"/>
-    <row r="125" ht="16" customHeight="1" s="53"/>
-    <row r="126" ht="16" customHeight="1" s="53"/>
-    <row r="127" ht="16" customHeight="1" s="53"/>
-    <row r="128" ht="16" customHeight="1" s="53"/>
-    <row r="129" ht="16" customHeight="1" s="53"/>
-    <row r="130" ht="16" customHeight="1" s="53"/>
-    <row r="131" ht="16" customHeight="1" s="53"/>
-    <row r="132" ht="16" customHeight="1" s="53"/>
-    <row r="133" ht="16" customHeight="1" s="53"/>
-    <row r="134" ht="16" customHeight="1" s="53"/>
-    <row r="135" ht="16" customHeight="1" s="53"/>
-    <row r="136" ht="16" customHeight="1" s="53"/>
-    <row r="137" ht="16" customHeight="1" s="53"/>
-    <row r="138" ht="16" customHeight="1" s="53"/>
-    <row r="139" ht="16" customHeight="1" s="53"/>
-    <row r="140" ht="16" customHeight="1" s="53"/>
-    <row r="141" ht="16" customHeight="1" s="53"/>
-    <row r="142" ht="16" customHeight="1" s="53"/>
-    <row r="143" ht="16" customHeight="1" s="53"/>
-    <row r="144" ht="16" customHeight="1" s="53"/>
-    <row r="145" ht="16" customHeight="1" s="53"/>
-    <row r="146" ht="16" customHeight="1" s="53"/>
-    <row r="147" ht="16" customHeight="1" s="53"/>
-    <row r="148" ht="16" customHeight="1" s="53"/>
-    <row r="149" ht="16" customHeight="1" s="53"/>
-    <row r="150" ht="16" customHeight="1" s="53"/>
-    <row r="151" ht="16" customHeight="1" s="53"/>
-    <row r="152" ht="16" customHeight="1" s="53"/>
-    <row r="153" ht="16" customHeight="1" s="53"/>
-    <row r="154" ht="16" customHeight="1" s="53"/>
-    <row r="155" ht="16" customHeight="1" s="53"/>
-    <row r="156" ht="16" customHeight="1" s="53"/>
-    <row r="157" ht="16" customHeight="1" s="53"/>
-    <row r="158" ht="16" customHeight="1" s="53"/>
-    <row r="159" ht="16" customHeight="1" s="53"/>
-    <row r="160" ht="16" customHeight="1" s="53"/>
-    <row r="161" ht="16" customHeight="1" s="53"/>
-    <row r="162" ht="16" customHeight="1" s="53"/>
-    <row r="163" ht="16" customHeight="1" s="53"/>
-    <row r="164" ht="16" customHeight="1" s="53"/>
-    <row r="165" ht="16" customHeight="1" s="53"/>
-    <row r="166" ht="16" customHeight="1" s="53"/>
-    <row r="167" ht="16" customHeight="1" s="53"/>
-    <row r="168" ht="16" customHeight="1" s="53"/>
-    <row r="169" ht="16" customHeight="1" s="53"/>
-    <row r="170" ht="16" customHeight="1" s="53"/>
-    <row r="171" ht="16" customHeight="1" s="53"/>
-    <row r="172" ht="16" customHeight="1" s="53"/>
-    <row r="173" ht="16" customHeight="1" s="53"/>
-    <row r="174" ht="16" customHeight="1" s="53"/>
-    <row r="175" ht="16" customHeight="1" s="53"/>
-    <row r="176" ht="16" customHeight="1" s="53"/>
-    <row r="177" ht="16" customHeight="1" s="53"/>
-    <row r="178" ht="16" customHeight="1" s="53"/>
-    <row r="179" ht="16" customHeight="1" s="53"/>
-    <row r="180" ht="16" customHeight="1" s="53"/>
-    <row r="181" ht="16" customHeight="1" s="53"/>
-    <row r="182" ht="16" customHeight="1" s="53"/>
-    <row r="183" ht="16" customHeight="1" s="53"/>
-    <row r="184" ht="16" customHeight="1" s="53"/>
-    <row r="185" ht="16" customHeight="1" s="53"/>
-    <row r="186" ht="16" customHeight="1" s="53"/>
-    <row r="187" ht="16" customHeight="1" s="53"/>
-    <row r="188" ht="16" customHeight="1" s="53"/>
-    <row r="189" ht="16" customHeight="1" s="53"/>
-    <row r="190" ht="16" customHeight="1" s="53"/>
-    <row r="191" ht="16" customHeight="1" s="53"/>
-    <row r="192" ht="16" customHeight="1" s="53"/>
-    <row r="193" ht="16" customHeight="1" s="53"/>
-    <row r="194" ht="16" customHeight="1" s="53"/>
-    <row r="195" ht="16" customHeight="1" s="53"/>
-    <row r="196" ht="16" customHeight="1" s="53"/>
-    <row r="197" ht="16" customHeight="1" s="53"/>
-    <row r="198" ht="16" customHeight="1" s="53"/>
-    <row r="199" ht="16" customHeight="1" s="53"/>
-    <row r="200" ht="16" customHeight="1" s="53"/>
-    <row r="201" ht="16" customHeight="1" s="53"/>
-    <row r="202" ht="16" customHeight="1" s="53"/>
-    <row r="203" ht="16" customHeight="1" s="53"/>
-    <row r="204" ht="16" customHeight="1" s="53"/>
-    <row r="205" ht="16" customHeight="1" s="53"/>
-    <row r="206" ht="16" customHeight="1" s="53"/>
-    <row r="207" ht="16" customHeight="1" s="53"/>
-    <row r="208" ht="16" customHeight="1" s="53"/>
-    <row r="209" ht="16" customHeight="1" s="53"/>
-    <row r="210" ht="16" customHeight="1" s="53"/>
-    <row r="211" ht="16" customHeight="1" s="53"/>
-    <row r="212" ht="16" customHeight="1" s="53"/>
-    <row r="213" ht="16" customHeight="1" s="53"/>
-    <row r="214" ht="16" customHeight="1" s="53"/>
-    <row r="215" ht="16" customHeight="1" s="53"/>
-    <row r="216" ht="16" customHeight="1" s="53"/>
-    <row r="217" ht="16" customHeight="1" s="53"/>
-    <row r="218" ht="16" customHeight="1" s="53"/>
-    <row r="219" ht="16" customHeight="1" s="53"/>
-    <row r="220" ht="16" customHeight="1" s="53"/>
-    <row r="221" ht="16" customHeight="1" s="53"/>
-    <row r="222" ht="16" customHeight="1" s="53"/>
-    <row r="223" ht="16" customHeight="1" s="53"/>
-    <row r="224" ht="16" customHeight="1" s="53"/>
-    <row r="225" ht="16" customHeight="1" s="53"/>
-    <row r="226" ht="16" customHeight="1" s="53"/>
-    <row r="227" ht="16" customHeight="1" s="53"/>
-    <row r="228" ht="16" customHeight="1" s="53"/>
-    <row r="229" ht="16" customHeight="1" s="53"/>
-    <row r="230" ht="16" customHeight="1" s="53"/>
-    <row r="231" ht="16" customHeight="1" s="53"/>
-    <row r="232" ht="16" customHeight="1" s="53"/>
-    <row r="233" ht="16" customHeight="1" s="53"/>
-    <row r="234" ht="16" customHeight="1" s="53"/>
-    <row r="235" ht="16" customHeight="1" s="53"/>
-    <row r="236" ht="16" customHeight="1" s="53"/>
-    <row r="237" ht="16" customHeight="1" s="53"/>
-    <row r="238" ht="16" customHeight="1" s="53"/>
-    <row r="239" ht="16" customHeight="1" s="53"/>
-    <row r="240" ht="16" customHeight="1" s="53"/>
-    <row r="241" ht="16" customHeight="1" s="53"/>
-    <row r="242" ht="16" customHeight="1" s="53"/>
-    <row r="243" ht="16" customHeight="1" s="53"/>
-    <row r="244" ht="16" customHeight="1" s="53"/>
-    <row r="245" ht="16" customHeight="1" s="53"/>
-    <row r="246" ht="16" customHeight="1" s="53"/>
-    <row r="247" ht="16" customHeight="1" s="53"/>
-    <row r="248" ht="16" customHeight="1" s="53"/>
-    <row r="249" ht="16" customHeight="1" s="53"/>
-    <row r="250" ht="16" customHeight="1" s="53"/>
-    <row r="251" ht="16" customHeight="1" s="53"/>
-    <row r="252" ht="16" customHeight="1" s="53"/>
-    <row r="253" ht="16" customHeight="1" s="53"/>
-    <row r="254" ht="16" customHeight="1" s="53"/>
-    <row r="255" ht="16" customHeight="1" s="53"/>
-    <row r="256" ht="16" customHeight="1" s="53"/>
-    <row r="257" ht="16" customHeight="1" s="53"/>
-    <row r="258" ht="16" customHeight="1" s="53"/>
-    <row r="259" ht="16" customHeight="1" s="53"/>
-    <row r="260" ht="16" customHeight="1" s="53"/>
-    <row r="261" ht="16" customHeight="1" s="53"/>
-    <row r="262" ht="16" customHeight="1" s="53"/>
+    <row customHeight="1" ht="16" r="65" s="53"/>
+    <row customHeight="1" ht="16" r="66" s="53"/>
+    <row customHeight="1" ht="16" r="67" s="53"/>
+    <row customHeight="1" ht="16" r="68" s="53"/>
+    <row customHeight="1" ht="16" r="69" s="53"/>
+    <row customHeight="1" ht="16" r="70" s="53"/>
+    <row customHeight="1" ht="16" r="71" s="53"/>
+    <row customHeight="1" ht="16" r="72" s="53"/>
+    <row customHeight="1" ht="16" r="73" s="53"/>
+    <row customHeight="1" ht="16" r="74" s="53"/>
+    <row customHeight="1" ht="16" r="75" s="53"/>
+    <row customHeight="1" ht="16" r="76" s="53"/>
+    <row customHeight="1" ht="16" r="77" s="53"/>
+    <row customHeight="1" ht="16" r="78" s="53"/>
+    <row customHeight="1" ht="16" r="79" s="53"/>
+    <row customHeight="1" ht="16" r="80" s="53"/>
+    <row customHeight="1" ht="16" r="81" s="53"/>
+    <row customHeight="1" ht="16" r="82" s="53"/>
+    <row customHeight="1" ht="16" r="83" s="53"/>
+    <row customHeight="1" ht="16" r="84" s="53"/>
+    <row customHeight="1" ht="16" r="85" s="53"/>
+    <row customHeight="1" ht="16" r="86" s="53"/>
+    <row customHeight="1" ht="16" r="87" s="53"/>
+    <row customHeight="1" ht="16" r="88" s="53"/>
+    <row customHeight="1" ht="16" r="89" s="53"/>
+    <row customHeight="1" ht="16" r="90" s="53"/>
+    <row customHeight="1" ht="16" r="91" s="53"/>
+    <row customHeight="1" ht="16" r="92" s="53"/>
+    <row customHeight="1" ht="16" r="93" s="53"/>
+    <row customHeight="1" ht="16" r="94" s="53"/>
+    <row customHeight="1" ht="16" r="95" s="53"/>
+    <row customHeight="1" ht="16" r="96" s="53"/>
+    <row customHeight="1" ht="16" r="97" s="53"/>
+    <row customHeight="1" ht="16" r="98" s="53"/>
+    <row customHeight="1" ht="16" r="99" s="53"/>
+    <row customHeight="1" ht="16" r="100" s="53"/>
+    <row customHeight="1" ht="16" r="101" s="53"/>
+    <row customHeight="1" ht="16" r="102" s="53"/>
+    <row customHeight="1" ht="16" r="103" s="53"/>
+    <row customHeight="1" ht="16" r="104" s="53"/>
+    <row customHeight="1" ht="16" r="105" s="53"/>
+    <row customHeight="1" ht="16" r="106" s="53"/>
+    <row customHeight="1" ht="16" r="107" s="53"/>
+    <row customHeight="1" ht="16" r="108" s="53"/>
+    <row customHeight="1" ht="16" r="109" s="53"/>
+    <row customHeight="1" ht="16" r="110" s="53"/>
+    <row customHeight="1" ht="16" r="111" s="53"/>
+    <row customHeight="1" ht="16" r="112" s="53"/>
+    <row customHeight="1" ht="16" r="113" s="53"/>
+    <row customHeight="1" ht="16" r="114" s="53"/>
+    <row customHeight="1" ht="16" r="115" s="53"/>
+    <row customHeight="1" ht="16" r="116" s="53"/>
+    <row customHeight="1" ht="16" r="117" s="53"/>
+    <row customHeight="1" ht="16" r="118" s="53"/>
+    <row customHeight="1" ht="16" r="119" s="53"/>
+    <row customHeight="1" ht="16" r="120" s="53"/>
+    <row customHeight="1" ht="16" r="121" s="53"/>
+    <row customHeight="1" ht="16" r="122" s="53"/>
+    <row customHeight="1" ht="16" r="123" s="53"/>
+    <row customHeight="1" ht="16" r="124" s="53"/>
+    <row customHeight="1" ht="16" r="125" s="53"/>
+    <row customHeight="1" ht="16" r="126" s="53"/>
+    <row customHeight="1" ht="16" r="127" s="53"/>
+    <row customHeight="1" ht="16" r="128" s="53"/>
+    <row customHeight="1" ht="16" r="129" s="53"/>
+    <row customHeight="1" ht="16" r="130" s="53"/>
+    <row customHeight="1" ht="16" r="131" s="53"/>
+    <row customHeight="1" ht="16" r="132" s="53"/>
+    <row customHeight="1" ht="16" r="133" s="53"/>
+    <row customHeight="1" ht="16" r="134" s="53"/>
+    <row customHeight="1" ht="16" r="135" s="53"/>
+    <row customHeight="1" ht="16" r="136" s="53"/>
+    <row customHeight="1" ht="16" r="137" s="53"/>
+    <row customHeight="1" ht="16" r="138" s="53"/>
+    <row customHeight="1" ht="16" r="139" s="53"/>
+    <row customHeight="1" ht="16" r="140" s="53"/>
+    <row customHeight="1" ht="16" r="141" s="53"/>
+    <row customHeight="1" ht="16" r="142" s="53"/>
+    <row customHeight="1" ht="16" r="143" s="53"/>
+    <row customHeight="1" ht="16" r="144" s="53"/>
+    <row customHeight="1" ht="16" r="145" s="53"/>
+    <row customHeight="1" ht="16" r="146" s="53"/>
+    <row customHeight="1" ht="16" r="147" s="53"/>
+    <row customHeight="1" ht="16" r="148" s="53"/>
+    <row customHeight="1" ht="16" r="149" s="53"/>
+    <row customHeight="1" ht="16" r="150" s="53"/>
+    <row customHeight="1" ht="16" r="151" s="53"/>
+    <row customHeight="1" ht="16" r="152" s="53"/>
+    <row customHeight="1" ht="16" r="153" s="53"/>
+    <row customHeight="1" ht="16" r="154" s="53"/>
+    <row customHeight="1" ht="16" r="155" s="53"/>
+    <row customHeight="1" ht="16" r="156" s="53"/>
+    <row customHeight="1" ht="16" r="157" s="53"/>
+    <row customHeight="1" ht="16" r="158" s="53"/>
+    <row customHeight="1" ht="16" r="159" s="53"/>
+    <row customHeight="1" ht="16" r="160" s="53"/>
+    <row customHeight="1" ht="16" r="161" s="53"/>
+    <row customHeight="1" ht="16" r="162" s="53"/>
+    <row customHeight="1" ht="16" r="163" s="53"/>
+    <row customHeight="1" ht="16" r="164" s="53"/>
+    <row customHeight="1" ht="16" r="165" s="53"/>
+    <row customHeight="1" ht="16" r="166" s="53"/>
+    <row customHeight="1" ht="16" r="167" s="53"/>
+    <row customHeight="1" ht="16" r="168" s="53"/>
+    <row customHeight="1" ht="16" r="169" s="53"/>
+    <row customHeight="1" ht="16" r="170" s="53"/>
+    <row customHeight="1" ht="16" r="171" s="53"/>
+    <row customHeight="1" ht="16" r="172" s="53"/>
+    <row customHeight="1" ht="16" r="173" s="53"/>
+    <row customHeight="1" ht="16" r="174" s="53"/>
+    <row customHeight="1" ht="16" r="175" s="53"/>
+    <row customHeight="1" ht="16" r="176" s="53"/>
+    <row customHeight="1" ht="16" r="177" s="53"/>
+    <row customHeight="1" ht="16" r="178" s="53"/>
+    <row customHeight="1" ht="16" r="179" s="53"/>
+    <row customHeight="1" ht="16" r="180" s="53"/>
+    <row customHeight="1" ht="16" r="181" s="53"/>
+    <row customHeight="1" ht="16" r="182" s="53"/>
+    <row customHeight="1" ht="16" r="183" s="53"/>
+    <row customHeight="1" ht="16" r="184" s="53"/>
+    <row customHeight="1" ht="16" r="185" s="53"/>
+    <row customHeight="1" ht="16" r="186" s="53"/>
+    <row customHeight="1" ht="16" r="187" s="53"/>
+    <row customHeight="1" ht="16" r="188" s="53"/>
+    <row customHeight="1" ht="16" r="189" s="53"/>
+    <row customHeight="1" ht="16" r="190" s="53"/>
+    <row customHeight="1" ht="16" r="191" s="53"/>
+    <row customHeight="1" ht="16" r="192" s="53"/>
+    <row customHeight="1" ht="16" r="193" s="53"/>
+    <row customHeight="1" ht="16" r="194" s="53"/>
+    <row customHeight="1" ht="16" r="195" s="53"/>
+    <row customHeight="1" ht="16" r="196" s="53"/>
+    <row customHeight="1" ht="16" r="197" s="53"/>
+    <row customHeight="1" ht="16" r="198" s="53"/>
+    <row customHeight="1" ht="16" r="199" s="53"/>
+    <row customHeight="1" ht="16" r="200" s="53"/>
+    <row customHeight="1" ht="16" r="201" s="53"/>
+    <row customHeight="1" ht="16" r="202" s="53"/>
+    <row customHeight="1" ht="16" r="203" s="53"/>
+    <row customHeight="1" ht="16" r="204" s="53"/>
+    <row customHeight="1" ht="16" r="205" s="53"/>
+    <row customHeight="1" ht="16" r="206" s="53"/>
+    <row customHeight="1" ht="16" r="207" s="53"/>
+    <row customHeight="1" ht="16" r="208" s="53"/>
+    <row customHeight="1" ht="16" r="209" s="53"/>
+    <row customHeight="1" ht="16" r="210" s="53"/>
+    <row customHeight="1" ht="16" r="211" s="53"/>
+    <row customHeight="1" ht="16" r="212" s="53"/>
+    <row customHeight="1" ht="16" r="213" s="53"/>
+    <row customHeight="1" ht="16" r="214" s="53"/>
+    <row customHeight="1" ht="16" r="215" s="53"/>
+    <row customHeight="1" ht="16" r="216" s="53"/>
+    <row customHeight="1" ht="16" r="217" s="53"/>
+    <row customHeight="1" ht="16" r="218" s="53"/>
+    <row customHeight="1" ht="16" r="219" s="53"/>
+    <row customHeight="1" ht="16" r="220" s="53"/>
+    <row customHeight="1" ht="16" r="221" s="53"/>
+    <row customHeight="1" ht="16" r="222" s="53"/>
+    <row customHeight="1" ht="16" r="223" s="53"/>
+    <row customHeight="1" ht="16" r="224" s="53"/>
+    <row customHeight="1" ht="16" r="225" s="53"/>
+    <row customHeight="1" ht="16" r="226" s="53"/>
+    <row customHeight="1" ht="16" r="227" s="53"/>
+    <row customHeight="1" ht="16" r="228" s="53"/>
+    <row customHeight="1" ht="16" r="229" s="53"/>
+    <row customHeight="1" ht="16" r="230" s="53"/>
+    <row customHeight="1" ht="16" r="231" s="53"/>
+    <row customHeight="1" ht="16" r="232" s="53"/>
+    <row customHeight="1" ht="16" r="233" s="53"/>
+    <row customHeight="1" ht="16" r="234" s="53"/>
+    <row customHeight="1" ht="16" r="235" s="53"/>
+    <row customHeight="1" ht="16" r="236" s="53"/>
+    <row customHeight="1" ht="16" r="237" s="53"/>
+    <row customHeight="1" ht="16" r="238" s="53"/>
+    <row customHeight="1" ht="16" r="239" s="53"/>
+    <row customHeight="1" ht="16" r="240" s="53"/>
+    <row customHeight="1" ht="16" r="241" s="53"/>
+    <row customHeight="1" ht="16" r="242" s="53"/>
+    <row customHeight="1" ht="16" r="243" s="53"/>
+    <row customHeight="1" ht="16" r="244" s="53"/>
+    <row customHeight="1" ht="16" r="245" s="53"/>
+    <row customHeight="1" ht="16" r="246" s="53"/>
+    <row customHeight="1" ht="16" r="247" s="53"/>
+    <row customHeight="1" ht="16" r="248" s="53"/>
+    <row customHeight="1" ht="16" r="249" s="53"/>
+    <row customHeight="1" ht="16" r="250" s="53"/>
+    <row customHeight="1" ht="16" r="251" s="53"/>
+    <row customHeight="1" ht="16" r="252" s="53"/>
+    <row customHeight="1" ht="16" r="253" s="53"/>
+    <row customHeight="1" ht="16" r="254" s="53"/>
+    <row customHeight="1" ht="16" r="255" s="53"/>
+    <row customHeight="1" ht="16" r="256" s="53"/>
+    <row customHeight="1" ht="16" r="257" s="53"/>
+    <row customHeight="1" ht="16" r="258" s="53"/>
+    <row customHeight="1" ht="16" r="259" s="53"/>
+    <row customHeight="1" ht="16" r="260" s="53"/>
+    <row customHeight="1" ht="16" r="261" s="53"/>
+    <row customHeight="1" ht="16" r="262" s="53"/>
   </sheetData>
   <autoFilter ref="A2:F61"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -4840,17 +4852,17 @@
   <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -4873,7 +4885,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>区域</t>
@@ -4959,7 +4971,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5002,7 +5014,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5047,7 +5059,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5084,7 +5096,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5129,7 +5141,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5168,7 +5180,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5205,7 +5217,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5234,7 +5246,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5273,7 +5285,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5310,7 +5322,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5347,7 +5359,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5386,7 +5398,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5423,7 +5435,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5450,7 +5462,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="10" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5478,7 +5490,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5506,7 +5518,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5534,7 +5546,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5564,7 +5576,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5594,7 +5606,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5630,7 +5642,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5658,7 +5670,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5688,7 +5700,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5726,7 +5738,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5756,7 +5768,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5788,7 +5800,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5822,7 +5834,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5854,7 +5866,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5882,7 +5894,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5918,7 +5930,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5945,7 +5957,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="10" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5977,7 +5989,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6009,7 +6021,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6034,7 +6046,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6064,7 +6076,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6094,7 +6106,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6128,7 +6140,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6158,7 +6170,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6186,7 +6198,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6214,7 +6226,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6242,7 +6254,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6270,7 +6282,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6298,7 +6310,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6326,7 +6338,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6354,7 +6366,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6382,7 +6394,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6420,7 +6432,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6450,7 +6462,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6486,7 +6498,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6520,7 +6532,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6556,7 +6568,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6588,7 +6600,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -7236,7 +7248,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -7249,17 +7261,17 @@
   <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -7282,7 +7294,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>区域</t>
@@ -7368,7 +7380,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7414,7 +7426,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7451,7 +7463,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7497,7 +7509,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7543,7 +7555,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7591,7 +7603,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7628,7 +7640,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7665,7 +7677,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7713,7 +7725,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7759,7 +7771,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7796,7 +7808,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7833,7 +7845,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7879,7 +7891,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7907,7 +7919,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -7935,7 +7947,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -7963,7 +7975,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -7991,7 +8003,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8019,7 +8031,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8047,7 +8059,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8075,7 +8087,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8103,7 +8115,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8131,7 +8143,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8159,7 +8171,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8187,7 +8199,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8215,7 +8227,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8243,7 +8255,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8273,7 +8285,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8301,7 +8313,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8329,7 +8341,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8357,7 +8369,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8385,7 +8397,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8413,7 +8425,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8441,7 +8453,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8471,7 +8483,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8499,7 +8511,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8527,7 +8539,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8555,7 +8567,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8583,7 +8595,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8613,7 +8625,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8645,7 +8657,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8673,7 +8685,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8701,7 +8713,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8729,7 +8741,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8757,7 +8769,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8785,7 +8797,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8817,7 +8829,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8849,7 +8861,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9525,7 +9537,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -9536,16 +9548,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
@@ -9555,7 +9567,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -9600,7 +9612,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9646,7 +9658,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9691,7 +9703,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9740,7 +9752,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9789,7 +9801,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9831,7 +9843,7 @@
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="35" t="n"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9866,7 +9878,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9906,7 +9918,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9942,7 +9954,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -9978,7 +9990,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10014,7 +10026,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10055,7 +10067,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10086,7 +10098,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10108,7 +10120,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10125,7 +10137,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10142,7 +10154,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10164,7 +10176,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10181,7 +10193,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10199,7 +10211,7 @@
       </c>
       <c r="D20" s="39" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10221,7 +10233,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10243,7 +10255,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10265,7 +10277,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10287,7 +10299,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10305,7 +10317,7 @@
       </c>
       <c r="D25" s="36" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10327,7 +10339,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10349,7 +10361,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10371,7 +10383,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10393,7 +10405,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10415,7 +10427,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10437,7 +10449,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10464,7 +10476,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10486,7 +10498,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10508,7 +10520,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10530,7 +10542,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10552,7 +10564,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10574,7 +10586,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10596,7 +10608,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10613,7 +10625,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10635,7 +10647,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10653,7 +10665,7 @@
       </c>
       <c r="D41" s="46" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10675,7 +10687,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10693,7 +10705,7 @@
       </c>
       <c r="D43" s="46" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10711,7 +10723,7 @@
       </c>
       <c r="E44" s="46" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10733,7 +10745,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10755,7 +10767,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10777,7 +10789,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10799,7 +10811,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10821,7 +10833,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10844,7 +10856,7 @@
       </c>
       <c r="E50" s="49" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10866,7 +10878,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10888,7 +10900,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10910,7 +10922,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="55" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -10932,7 +10944,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="55" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10954,7 +10966,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10976,7 +10988,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10994,7 +11006,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -11005,18 +11017,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6.83203125" customWidth="1" style="23" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="23" min="2" max="2"/>
-    <col width="19.6640625" customWidth="1" style="23" min="3" max="3"/>
-    <col width="13" customWidth="1" style="23" min="4" max="4"/>
-    <col hidden="1" width="30.5" customWidth="1" style="23" min="5" max="6"/>
-    <col width="30.5" customWidth="1" style="23" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="23" min="8" max="26"/>
+    <col customWidth="1" max="1" min="1" style="23" width="6.83203125"/>
+    <col customWidth="1" max="2" min="2" style="23" width="8.83203125"/>
+    <col customWidth="1" max="3" min="3" style="23" width="19.6640625"/>
+    <col customWidth="1" max="4" min="4" style="23" width="13"/>
+    <col customWidth="1" hidden="1" max="6" min="5" style="23" width="30.5"/>
+    <col customWidth="1" max="7" min="7" style="23" width="30.5"/>
+    <col customWidth="1" max="26" min="8" style="23" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="1" s="53">
       <c r="A1" s="21" t="n"/>
       <c r="B1" s="22" t="inlineStr">
         <is>
@@ -11058,7 +11070,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="2" s="53">
       <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
@@ -11101,7 +11113,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="3" s="53">
       <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
@@ -11134,7 +11146,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="4" s="53">
       <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
@@ -11172,7 +11184,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="5" s="53">
       <c r="A5" s="24" t="n">
         <v>4</v>
       </c>
@@ -11215,7 +11227,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="6" s="53">
       <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
@@ -11248,7 +11260,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="7" s="53">
       <c r="A7" s="24" t="n">
         <v>6</v>
       </c>
@@ -11277,7 +11289,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="8" s="53">
       <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
@@ -11307,7 +11319,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="9" s="53">
       <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
@@ -11332,7 +11344,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="10" s="53">
       <c r="A10" s="24" t="n">
         <v>1</v>
       </c>
@@ -11357,7 +11369,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="11" s="53">
       <c r="A11" s="24" t="n">
         <v>2</v>
       </c>
@@ -11387,7 +11399,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="12" s="53">
       <c r="A12" s="24" t="n">
         <v>3</v>
       </c>
@@ -11412,7 +11424,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="13" s="53">
       <c r="A13" s="24" t="n">
         <v>4</v>
       </c>
@@ -11442,7 +11454,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="14" s="53">
       <c r="A14" s="24" t="n">
         <v>5</v>
       </c>
@@ -11462,7 +11474,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="15" s="53">
       <c r="A15" s="24" t="n">
         <v>6</v>
       </c>
@@ -11492,7 +11504,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="16" s="53">
       <c r="A16" s="24" t="n">
         <v>1</v>
       </c>
@@ -11517,7 +11529,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="17" s="53">
       <c r="A17" s="24" t="n">
         <v>2</v>
       </c>
@@ -11552,7 +11564,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="18" s="53">
       <c r="A18" s="24" t="n">
         <v>3</v>
       </c>
@@ -11587,7 +11599,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="19" s="53">
       <c r="A19" s="24" t="n">
         <v>4</v>
       </c>
@@ -11612,7 +11624,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="20" s="53">
       <c r="A20" s="24" t="n">
         <v>5</v>
       </c>
@@ -11642,7 +11654,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="21" s="53">
       <c r="A21" s="24" t="n">
         <v>6</v>
       </c>
@@ -11672,7 +11684,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="22" s="53">
       <c r="A22" s="24" t="n">
         <v>7</v>
       </c>
@@ -11702,7 +11714,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="23" s="53">
       <c r="A23" s="24" t="n">
         <v>8</v>
       </c>
@@ -11732,7 +11744,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="24" s="53">
       <c r="A24" s="24" t="n">
         <v>1</v>
       </c>
@@ -11762,7 +11774,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="25" s="53">
       <c r="A25" s="24" t="n">
         <v>2</v>
       </c>
@@ -11792,7 +11804,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="26" s="53">
       <c r="A26" s="24" t="n">
         <v>3</v>
       </c>
@@ -11817,7 +11829,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="27" s="53">
       <c r="A27" s="24" t="n">
         <v>4</v>
       </c>
@@ -11847,7 +11859,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="28" s="53">
       <c r="A28" s="24" t="n">
         <v>5</v>
       </c>
@@ -11877,7 +11889,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="29" s="53">
       <c r="A29" s="24" t="n">
         <v>6</v>
       </c>
@@ -11907,7 +11919,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="30" s="53">
       <c r="A30" s="24" t="n">
         <v>7</v>
       </c>
@@ -11942,7 +11954,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="31" s="53">
       <c r="A31" s="24" t="n">
         <v>8</v>
       </c>
@@ -11972,7 +11984,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="32" s="53">
       <c r="A32" s="24" t="n">
         <v>1</v>
       </c>
@@ -12002,7 +12014,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="33" s="53">
       <c r="A33" s="24" t="n">
         <v>2</v>
       </c>
@@ -12032,7 +12044,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="34" s="53">
       <c r="A34" s="24" t="n">
         <v>3</v>
       </c>
@@ -12062,7 +12074,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="35" s="53">
       <c r="A35" s="24" t="n">
         <v>4</v>
       </c>
@@ -12092,7 +12104,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="36" s="53">
       <c r="A36" s="24" t="n">
         <v>1</v>
       </c>
@@ -12122,7 +12134,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="37" s="53">
       <c r="A37" s="24" t="n">
         <v>2</v>
       </c>
@@ -12157,7 +12169,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="38" s="53">
       <c r="A38" s="24" t="n">
         <v>3</v>
       </c>
@@ -12188,6 +12200,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
report: update 2026-07-29 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46229</v>
+        <v>46232</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="D34" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发1次</t>
+          <t>累计未发2次，迟发1次</t>
         </is>
       </c>
       <c r="E34" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-02 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46232</v>
+        <v>46236</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发4次</t>
+          <t>累计未发2次，迟发4次</t>
         </is>
       </c>
       <c r="E10" s="69" t="n"/>
@@ -4194,7 +4194,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D48" s="71" t="n"/>
+      <c r="D48" s="71" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E48" s="69" t="n"/>
       <c r="F48" s="63" t="inlineStr">
         <is>
@@ -4495,7 +4499,7 @@
       </c>
       <c r="D59" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发1次</t>
+          <t>累计未发1次，迟发2次</t>
         </is>
       </c>
       <c r="E59" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-05 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46236</v>
+        <v>46239</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="D26" s="68" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E26" s="69" t="n"/>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="D27" s="71" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E27" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-09 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46239</v>
+        <v>46243</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2764,7 +2764,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D4" s="71" t="n"/>
+      <c r="D4" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E4" s="69" t="n"/>
       <c r="F4" s="63" t="inlineStr">
         <is>
@@ -4059,7 +4063,7 @@
       </c>
       <c r="D43" s="68" t="inlineStr">
         <is>
-          <t>迟发2次</t>
+          <t>累计未发1次，迟发2次</t>
         </is>
       </c>
       <c r="E43" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-10 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="D30" s="68" t="inlineStr">
         <is>
-          <t>迟发3次</t>
+          <t>累计未发1次，迟发3次</t>
         </is>
       </c>
       <c r="E30" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-11 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="D4" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E4" s="69" t="n"/>
@@ -3679,7 +3679,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D29" s="70" t="n"/>
+      <c r="D29" s="70" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E29" s="69" t="n"/>
       <c r="F29" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-08-16 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="27040" windowHeight="16400" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16400" windowWidth="27040" xWindow="0" yWindow="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026年日报'!$A$2:$F$61</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'2026年日报'!$A$2:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,257 +449,257 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1">
+    <xf applyAlignment="1" borderId="7" fillId="7" fontId="0" numFmtId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="83">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="3" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="5" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="5" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="10" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="11" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="12" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="16" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="14" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="9" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -1073,16 +1073,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1557,7 +1557,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1642,7 +1642,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D40" s="46" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D48" s="51" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -2619,26 +2619,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O65"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46245</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+        <v>46250</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>区域</t>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2812,7 +2812,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2876,7 +2876,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2931,7 +2931,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="72" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -2982,7 +2982,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3028,7 +3028,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3070,7 +3070,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -3116,7 +3116,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3162,7 +3162,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3204,7 +3204,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3246,7 +3246,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3283,7 +3283,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="15" s="78">
       <c r="A15" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3314,7 +3314,7 @@
       <c r="H15" s="23" t="n"/>
       <c r="J15" s="67" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="G17" s="67" t="n"/>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="G18" s="67" t="n"/>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="61" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="G19" s="67" t="n"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="G20" s="67" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="G21" s="67" t="n"/>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="G22" s="67" t="n"/>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="G23" s="67" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="G24" s="67" t="n"/>
     </row>
-    <row r="25" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="25" s="78">
       <c r="A25" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3578,7 +3578,7 @@
       <c r="H25" s="67" t="n"/>
       <c r="J25" s="67" t="n"/>
     </row>
-    <row r="26" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="26" s="78">
       <c r="A26" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3609,7 +3609,7 @@
       <c r="H26" s="67" t="n"/>
       <c r="J26" s="67" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="G27" s="67" t="n"/>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3663,7 +3663,7 @@
       </c>
       <c r="G28" s="67" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -3692,7 +3692,7 @@
       </c>
       <c r="G29" s="67" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="G30" s="67" t="n"/>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="G31" s="67" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="61" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="G32" s="67" t="n"/>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3800,7 +3800,7 @@
       </c>
       <c r="G33" s="67" t="n"/>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="G34" s="67" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="G35" s="67" t="n"/>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="G36" s="67" t="n"/>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="G37" s="67" t="n"/>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="G38" s="67" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="G39" s="67" t="n"/>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="G40" s="67" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="G41" s="67" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="G42" s="67" t="n"/>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="G43" s="67" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="G44" s="67" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="G45" s="67" t="n"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="G46" s="67" t="n"/>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="G47" s="67" t="n"/>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="61" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -4215,7 +4215,7 @@
       </c>
       <c r="G48" s="67" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="G49" s="67" t="n"/>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="G50" s="67" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4285,7 +4285,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D51" s="71" t="n"/>
+      <c r="D51" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E51" s="69" t="n"/>
       <c r="F51" s="63" t="inlineStr">
         <is>
@@ -4294,7 +4298,7 @@
       </c>
       <c r="G51" s="67" t="n"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4319,7 +4323,7 @@
       </c>
       <c r="G52" s="67" t="n"/>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="72" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -4348,7 +4352,7 @@
       </c>
       <c r="G53" s="67" t="n"/>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="58" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -4377,7 +4381,7 @@
       </c>
       <c r="G54" s="67" t="n"/>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4406,7 +4410,7 @@
       </c>
       <c r="G55" s="67" t="n"/>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4431,7 +4435,7 @@
       </c>
       <c r="G56" s="67" t="n"/>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="58" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -4460,7 +4464,7 @@
       </c>
       <c r="G57" s="67" t="n"/>
     </row>
-    <row r="58" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="58" s="53">
       <c r="A58" s="60" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4478,7 +4482,7 @@
       </c>
       <c r="D58" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E58" s="69" t="n"/>
@@ -4489,7 +4493,7 @@
       </c>
       <c r="G58" s="67" t="n"/>
     </row>
-    <row r="59" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="59" s="53">
       <c r="A59" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4518,7 +4522,7 @@
       </c>
       <c r="G59" s="67" t="n"/>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="60" s="53">
       <c r="A60" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4543,7 +4547,7 @@
       </c>
       <c r="G60" s="67" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="61" s="53">
       <c r="A61" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4572,7 +4576,7 @@
       </c>
       <c r="G61" s="67" t="n"/>
     </row>
-    <row r="62" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="62" s="53">
       <c r="A62" s="60" t="inlineStr">
         <is>
           <t>粤西五区</t>
@@ -4596,7 +4600,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="63" s="53">
       <c r="A63" s="60" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -4624,7 +4628,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="64" s="53">
       <c r="A64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4651,228 +4655,228 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1" s="53">
-      <c r="A65" t="inlineStr">
+    <row customHeight="1" ht="16" r="65" s="53">
+      <c r="A65" s="0" t="inlineStr">
         <is>
           <t>华东分公司</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="0" t="inlineStr">
         <is>
           <t>南京江宁中心</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F65" s="0" t="inlineStr">
         <is>
           <t>华东分公司</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1" s="53"/>
-    <row r="67" ht="16" customHeight="1" s="53"/>
-    <row r="68" ht="16" customHeight="1" s="53"/>
-    <row r="69" ht="16" customHeight="1" s="53"/>
-    <row r="70" ht="16" customHeight="1" s="53"/>
-    <row r="71" ht="16" customHeight="1" s="53"/>
-    <row r="72" ht="16" customHeight="1" s="53"/>
-    <row r="73" ht="16" customHeight="1" s="53"/>
-    <row r="74" ht="16" customHeight="1" s="53"/>
-    <row r="75" ht="16" customHeight="1" s="53"/>
-    <row r="76" ht="16" customHeight="1" s="53"/>
-    <row r="77" ht="16" customHeight="1" s="53"/>
-    <row r="78" ht="16" customHeight="1" s="53"/>
-    <row r="79" ht="16" customHeight="1" s="53"/>
-    <row r="80" ht="16" customHeight="1" s="53"/>
-    <row r="81" ht="16" customHeight="1" s="53"/>
-    <row r="82" ht="16" customHeight="1" s="53"/>
-    <row r="83" ht="16" customHeight="1" s="53"/>
-    <row r="84" ht="16" customHeight="1" s="53"/>
-    <row r="85" ht="16" customHeight="1" s="53"/>
-    <row r="86" ht="16" customHeight="1" s="53"/>
-    <row r="87" ht="16" customHeight="1" s="53"/>
-    <row r="88" ht="16" customHeight="1" s="53"/>
-    <row r="89" ht="16" customHeight="1" s="53"/>
-    <row r="90" ht="16" customHeight="1" s="53"/>
-    <row r="91" ht="16" customHeight="1" s="53"/>
-    <row r="92" ht="16" customHeight="1" s="53"/>
-    <row r="93" ht="16" customHeight="1" s="53"/>
-    <row r="94" ht="16" customHeight="1" s="53"/>
-    <row r="95" ht="16" customHeight="1" s="53"/>
-    <row r="96" ht="16" customHeight="1" s="53"/>
-    <row r="97" ht="16" customHeight="1" s="53"/>
-    <row r="98" ht="16" customHeight="1" s="53"/>
-    <row r="99" ht="16" customHeight="1" s="53"/>
-    <row r="100" ht="16" customHeight="1" s="53"/>
-    <row r="101" ht="16" customHeight="1" s="53"/>
-    <row r="102" ht="16" customHeight="1" s="53"/>
-    <row r="103" ht="16" customHeight="1" s="53"/>
-    <row r="104" ht="16" customHeight="1" s="53"/>
-    <row r="105" ht="16" customHeight="1" s="53"/>
-    <row r="106" ht="16" customHeight="1" s="53"/>
-    <row r="107" ht="16" customHeight="1" s="53"/>
-    <row r="108" ht="16" customHeight="1" s="53"/>
-    <row r="109" ht="16" customHeight="1" s="53"/>
-    <row r="110" ht="16" customHeight="1" s="53"/>
-    <row r="111" ht="16" customHeight="1" s="53"/>
-    <row r="112" ht="16" customHeight="1" s="53"/>
-    <row r="113" ht="16" customHeight="1" s="53"/>
-    <row r="114" ht="16" customHeight="1" s="53"/>
-    <row r="115" ht="16" customHeight="1" s="53"/>
-    <row r="116" ht="16" customHeight="1" s="53"/>
-    <row r="117" ht="16" customHeight="1" s="53"/>
-    <row r="118" ht="16" customHeight="1" s="53"/>
-    <row r="119" ht="16" customHeight="1" s="53"/>
-    <row r="120" ht="16" customHeight="1" s="53"/>
-    <row r="121" ht="16" customHeight="1" s="53"/>
-    <row r="122" ht="16" customHeight="1" s="53"/>
-    <row r="123" ht="16" customHeight="1" s="53"/>
-    <row r="124" ht="16" customHeight="1" s="53"/>
-    <row r="125" ht="16" customHeight="1" s="53"/>
-    <row r="126" ht="16" customHeight="1" s="53"/>
-    <row r="127" ht="16" customHeight="1" s="53"/>
-    <row r="128" ht="16" customHeight="1" s="53"/>
-    <row r="129" ht="16" customHeight="1" s="53"/>
-    <row r="130" ht="16" customHeight="1" s="53"/>
-    <row r="131" ht="16" customHeight="1" s="53"/>
-    <row r="132" ht="16" customHeight="1" s="53"/>
-    <row r="133" ht="16" customHeight="1" s="53"/>
-    <row r="134" ht="16" customHeight="1" s="53"/>
-    <row r="135" ht="16" customHeight="1" s="53"/>
-    <row r="136" ht="16" customHeight="1" s="53"/>
-    <row r="137" ht="16" customHeight="1" s="53"/>
-    <row r="138" ht="16" customHeight="1" s="53"/>
-    <row r="139" ht="16" customHeight="1" s="53"/>
-    <row r="140" ht="16" customHeight="1" s="53"/>
-    <row r="141" ht="16" customHeight="1" s="53"/>
-    <row r="142" ht="16" customHeight="1" s="53"/>
-    <row r="143" ht="16" customHeight="1" s="53"/>
-    <row r="144" ht="16" customHeight="1" s="53"/>
-    <row r="145" ht="16" customHeight="1" s="53"/>
-    <row r="146" ht="16" customHeight="1" s="53"/>
-    <row r="147" ht="16" customHeight="1" s="53"/>
-    <row r="148" ht="16" customHeight="1" s="53"/>
-    <row r="149" ht="16" customHeight="1" s="53"/>
-    <row r="150" ht="16" customHeight="1" s="53"/>
-    <row r="151" ht="16" customHeight="1" s="53"/>
-    <row r="152" ht="16" customHeight="1" s="53"/>
-    <row r="153" ht="16" customHeight="1" s="53"/>
-    <row r="154" ht="16" customHeight="1" s="53"/>
-    <row r="155" ht="16" customHeight="1" s="53"/>
-    <row r="156" ht="16" customHeight="1" s="53"/>
-    <row r="157" ht="16" customHeight="1" s="53"/>
-    <row r="158" ht="16" customHeight="1" s="53"/>
-    <row r="159" ht="16" customHeight="1" s="53"/>
-    <row r="160" ht="16" customHeight="1" s="53"/>
-    <row r="161" ht="16" customHeight="1" s="53"/>
-    <row r="162" ht="16" customHeight="1" s="53"/>
-    <row r="163" ht="16" customHeight="1" s="53"/>
-    <row r="164" ht="16" customHeight="1" s="53"/>
-    <row r="165" ht="16" customHeight="1" s="53"/>
-    <row r="166" ht="16" customHeight="1" s="53"/>
-    <row r="167" ht="16" customHeight="1" s="53"/>
-    <row r="168" ht="16" customHeight="1" s="53"/>
-    <row r="169" ht="16" customHeight="1" s="53"/>
-    <row r="170" ht="16" customHeight="1" s="53"/>
-    <row r="171" ht="16" customHeight="1" s="53"/>
-    <row r="172" ht="16" customHeight="1" s="53"/>
-    <row r="173" ht="16" customHeight="1" s="53"/>
-    <row r="174" ht="16" customHeight="1" s="53"/>
-    <row r="175" ht="16" customHeight="1" s="53"/>
-    <row r="176" ht="16" customHeight="1" s="53"/>
-    <row r="177" ht="16" customHeight="1" s="53"/>
-    <row r="178" ht="16" customHeight="1" s="53"/>
-    <row r="179" ht="16" customHeight="1" s="53"/>
-    <row r="180" ht="16" customHeight="1" s="53"/>
-    <row r="181" ht="16" customHeight="1" s="53"/>
-    <row r="182" ht="16" customHeight="1" s="53"/>
-    <row r="183" ht="16" customHeight="1" s="53"/>
-    <row r="184" ht="16" customHeight="1" s="53"/>
-    <row r="185" ht="16" customHeight="1" s="53"/>
-    <row r="186" ht="16" customHeight="1" s="53"/>
-    <row r="187" ht="16" customHeight="1" s="53"/>
-    <row r="188" ht="16" customHeight="1" s="53"/>
-    <row r="189" ht="16" customHeight="1" s="53"/>
-    <row r="190" ht="16" customHeight="1" s="53"/>
-    <row r="191" ht="16" customHeight="1" s="53"/>
-    <row r="192" ht="16" customHeight="1" s="53"/>
-    <row r="193" ht="16" customHeight="1" s="53"/>
-    <row r="194" ht="16" customHeight="1" s="53"/>
-    <row r="195" ht="16" customHeight="1" s="53"/>
-    <row r="196" ht="16" customHeight="1" s="53"/>
-    <row r="197" ht="16" customHeight="1" s="53"/>
-    <row r="198" ht="16" customHeight="1" s="53"/>
-    <row r="199" ht="16" customHeight="1" s="53"/>
-    <row r="200" ht="16" customHeight="1" s="53"/>
-    <row r="201" ht="16" customHeight="1" s="53"/>
-    <row r="202" ht="16" customHeight="1" s="53"/>
-    <row r="203" ht="16" customHeight="1" s="53"/>
-    <row r="204" ht="16" customHeight="1" s="53"/>
-    <row r="205" ht="16" customHeight="1" s="53"/>
-    <row r="206" ht="16" customHeight="1" s="53"/>
-    <row r="207" ht="16" customHeight="1" s="53"/>
-    <row r="208" ht="16" customHeight="1" s="53"/>
-    <row r="209" ht="16" customHeight="1" s="53"/>
-    <row r="210" ht="16" customHeight="1" s="53"/>
-    <row r="211" ht="16" customHeight="1" s="53"/>
-    <row r="212" ht="16" customHeight="1" s="53"/>
-    <row r="213" ht="16" customHeight="1" s="53"/>
-    <row r="214" ht="16" customHeight="1" s="53"/>
-    <row r="215" ht="16" customHeight="1" s="53"/>
-    <row r="216" ht="16" customHeight="1" s="53"/>
-    <row r="217" ht="16" customHeight="1" s="53"/>
-    <row r="218" ht="16" customHeight="1" s="53"/>
-    <row r="219" ht="16" customHeight="1" s="53"/>
-    <row r="220" ht="16" customHeight="1" s="53"/>
-    <row r="221" ht="16" customHeight="1" s="53"/>
-    <row r="222" ht="16" customHeight="1" s="53"/>
-    <row r="223" ht="16" customHeight="1" s="53"/>
-    <row r="224" ht="16" customHeight="1" s="53"/>
-    <row r="225" ht="16" customHeight="1" s="53"/>
-    <row r="226" ht="16" customHeight="1" s="53"/>
-    <row r="227" ht="16" customHeight="1" s="53"/>
-    <row r="228" ht="16" customHeight="1" s="53"/>
-    <row r="229" ht="16" customHeight="1" s="53"/>
-    <row r="230" ht="16" customHeight="1" s="53"/>
-    <row r="231" ht="16" customHeight="1" s="53"/>
-    <row r="232" ht="16" customHeight="1" s="53"/>
-    <row r="233" ht="16" customHeight="1" s="53"/>
-    <row r="234" ht="16" customHeight="1" s="53"/>
-    <row r="235" ht="16" customHeight="1" s="53"/>
-    <row r="236" ht="16" customHeight="1" s="53"/>
-    <row r="237" ht="16" customHeight="1" s="53"/>
-    <row r="238" ht="16" customHeight="1" s="53"/>
-    <row r="239" ht="16" customHeight="1" s="53"/>
-    <row r="240" ht="16" customHeight="1" s="53"/>
-    <row r="241" ht="16" customHeight="1" s="53"/>
-    <row r="242" ht="16" customHeight="1" s="53"/>
-    <row r="243" ht="16" customHeight="1" s="53"/>
-    <row r="244" ht="16" customHeight="1" s="53"/>
-    <row r="245" ht="16" customHeight="1" s="53"/>
-    <row r="246" ht="16" customHeight="1" s="53"/>
-    <row r="247" ht="16" customHeight="1" s="53"/>
-    <row r="248" ht="16" customHeight="1" s="53"/>
-    <row r="249" ht="16" customHeight="1" s="53"/>
-    <row r="250" ht="16" customHeight="1" s="53"/>
-    <row r="251" ht="16" customHeight="1" s="53"/>
-    <row r="252" ht="16" customHeight="1" s="53"/>
-    <row r="253" ht="16" customHeight="1" s="53"/>
-    <row r="254" ht="16" customHeight="1" s="53"/>
-    <row r="255" ht="16" customHeight="1" s="53"/>
-    <row r="256" ht="16" customHeight="1" s="53"/>
-    <row r="257" ht="16" customHeight="1" s="53"/>
-    <row r="258" ht="16" customHeight="1" s="53"/>
-    <row r="259" ht="16" customHeight="1" s="53"/>
-    <row r="260" ht="16" customHeight="1" s="53"/>
-    <row r="261" ht="16" customHeight="1" s="53"/>
-    <row r="262" ht="16" customHeight="1" s="53"/>
+    <row customHeight="1" ht="16" r="66" s="53"/>
+    <row customHeight="1" ht="16" r="67" s="53"/>
+    <row customHeight="1" ht="16" r="68" s="53"/>
+    <row customHeight="1" ht="16" r="69" s="53"/>
+    <row customHeight="1" ht="16" r="70" s="53"/>
+    <row customHeight="1" ht="16" r="71" s="53"/>
+    <row customHeight="1" ht="16" r="72" s="53"/>
+    <row customHeight="1" ht="16" r="73" s="53"/>
+    <row customHeight="1" ht="16" r="74" s="53"/>
+    <row customHeight="1" ht="16" r="75" s="53"/>
+    <row customHeight="1" ht="16" r="76" s="53"/>
+    <row customHeight="1" ht="16" r="77" s="53"/>
+    <row customHeight="1" ht="16" r="78" s="53"/>
+    <row customHeight="1" ht="16" r="79" s="53"/>
+    <row customHeight="1" ht="16" r="80" s="53"/>
+    <row customHeight="1" ht="16" r="81" s="53"/>
+    <row customHeight="1" ht="16" r="82" s="53"/>
+    <row customHeight="1" ht="16" r="83" s="53"/>
+    <row customHeight="1" ht="16" r="84" s="53"/>
+    <row customHeight="1" ht="16" r="85" s="53"/>
+    <row customHeight="1" ht="16" r="86" s="53"/>
+    <row customHeight="1" ht="16" r="87" s="53"/>
+    <row customHeight="1" ht="16" r="88" s="53"/>
+    <row customHeight="1" ht="16" r="89" s="53"/>
+    <row customHeight="1" ht="16" r="90" s="53"/>
+    <row customHeight="1" ht="16" r="91" s="53"/>
+    <row customHeight="1" ht="16" r="92" s="53"/>
+    <row customHeight="1" ht="16" r="93" s="53"/>
+    <row customHeight="1" ht="16" r="94" s="53"/>
+    <row customHeight="1" ht="16" r="95" s="53"/>
+    <row customHeight="1" ht="16" r="96" s="53"/>
+    <row customHeight="1" ht="16" r="97" s="53"/>
+    <row customHeight="1" ht="16" r="98" s="53"/>
+    <row customHeight="1" ht="16" r="99" s="53"/>
+    <row customHeight="1" ht="16" r="100" s="53"/>
+    <row customHeight="1" ht="16" r="101" s="53"/>
+    <row customHeight="1" ht="16" r="102" s="53"/>
+    <row customHeight="1" ht="16" r="103" s="53"/>
+    <row customHeight="1" ht="16" r="104" s="53"/>
+    <row customHeight="1" ht="16" r="105" s="53"/>
+    <row customHeight="1" ht="16" r="106" s="53"/>
+    <row customHeight="1" ht="16" r="107" s="53"/>
+    <row customHeight="1" ht="16" r="108" s="53"/>
+    <row customHeight="1" ht="16" r="109" s="53"/>
+    <row customHeight="1" ht="16" r="110" s="53"/>
+    <row customHeight="1" ht="16" r="111" s="53"/>
+    <row customHeight="1" ht="16" r="112" s="53"/>
+    <row customHeight="1" ht="16" r="113" s="53"/>
+    <row customHeight="1" ht="16" r="114" s="53"/>
+    <row customHeight="1" ht="16" r="115" s="53"/>
+    <row customHeight="1" ht="16" r="116" s="53"/>
+    <row customHeight="1" ht="16" r="117" s="53"/>
+    <row customHeight="1" ht="16" r="118" s="53"/>
+    <row customHeight="1" ht="16" r="119" s="53"/>
+    <row customHeight="1" ht="16" r="120" s="53"/>
+    <row customHeight="1" ht="16" r="121" s="53"/>
+    <row customHeight="1" ht="16" r="122" s="53"/>
+    <row customHeight="1" ht="16" r="123" s="53"/>
+    <row customHeight="1" ht="16" r="124" s="53"/>
+    <row customHeight="1" ht="16" r="125" s="53"/>
+    <row customHeight="1" ht="16" r="126" s="53"/>
+    <row customHeight="1" ht="16" r="127" s="53"/>
+    <row customHeight="1" ht="16" r="128" s="53"/>
+    <row customHeight="1" ht="16" r="129" s="53"/>
+    <row customHeight="1" ht="16" r="130" s="53"/>
+    <row customHeight="1" ht="16" r="131" s="53"/>
+    <row customHeight="1" ht="16" r="132" s="53"/>
+    <row customHeight="1" ht="16" r="133" s="53"/>
+    <row customHeight="1" ht="16" r="134" s="53"/>
+    <row customHeight="1" ht="16" r="135" s="53"/>
+    <row customHeight="1" ht="16" r="136" s="53"/>
+    <row customHeight="1" ht="16" r="137" s="53"/>
+    <row customHeight="1" ht="16" r="138" s="53"/>
+    <row customHeight="1" ht="16" r="139" s="53"/>
+    <row customHeight="1" ht="16" r="140" s="53"/>
+    <row customHeight="1" ht="16" r="141" s="53"/>
+    <row customHeight="1" ht="16" r="142" s="53"/>
+    <row customHeight="1" ht="16" r="143" s="53"/>
+    <row customHeight="1" ht="16" r="144" s="53"/>
+    <row customHeight="1" ht="16" r="145" s="53"/>
+    <row customHeight="1" ht="16" r="146" s="53"/>
+    <row customHeight="1" ht="16" r="147" s="53"/>
+    <row customHeight="1" ht="16" r="148" s="53"/>
+    <row customHeight="1" ht="16" r="149" s="53"/>
+    <row customHeight="1" ht="16" r="150" s="53"/>
+    <row customHeight="1" ht="16" r="151" s="53"/>
+    <row customHeight="1" ht="16" r="152" s="53"/>
+    <row customHeight="1" ht="16" r="153" s="53"/>
+    <row customHeight="1" ht="16" r="154" s="53"/>
+    <row customHeight="1" ht="16" r="155" s="53"/>
+    <row customHeight="1" ht="16" r="156" s="53"/>
+    <row customHeight="1" ht="16" r="157" s="53"/>
+    <row customHeight="1" ht="16" r="158" s="53"/>
+    <row customHeight="1" ht="16" r="159" s="53"/>
+    <row customHeight="1" ht="16" r="160" s="53"/>
+    <row customHeight="1" ht="16" r="161" s="53"/>
+    <row customHeight="1" ht="16" r="162" s="53"/>
+    <row customHeight="1" ht="16" r="163" s="53"/>
+    <row customHeight="1" ht="16" r="164" s="53"/>
+    <row customHeight="1" ht="16" r="165" s="53"/>
+    <row customHeight="1" ht="16" r="166" s="53"/>
+    <row customHeight="1" ht="16" r="167" s="53"/>
+    <row customHeight="1" ht="16" r="168" s="53"/>
+    <row customHeight="1" ht="16" r="169" s="53"/>
+    <row customHeight="1" ht="16" r="170" s="53"/>
+    <row customHeight="1" ht="16" r="171" s="53"/>
+    <row customHeight="1" ht="16" r="172" s="53"/>
+    <row customHeight="1" ht="16" r="173" s="53"/>
+    <row customHeight="1" ht="16" r="174" s="53"/>
+    <row customHeight="1" ht="16" r="175" s="53"/>
+    <row customHeight="1" ht="16" r="176" s="53"/>
+    <row customHeight="1" ht="16" r="177" s="53"/>
+    <row customHeight="1" ht="16" r="178" s="53"/>
+    <row customHeight="1" ht="16" r="179" s="53"/>
+    <row customHeight="1" ht="16" r="180" s="53"/>
+    <row customHeight="1" ht="16" r="181" s="53"/>
+    <row customHeight="1" ht="16" r="182" s="53"/>
+    <row customHeight="1" ht="16" r="183" s="53"/>
+    <row customHeight="1" ht="16" r="184" s="53"/>
+    <row customHeight="1" ht="16" r="185" s="53"/>
+    <row customHeight="1" ht="16" r="186" s="53"/>
+    <row customHeight="1" ht="16" r="187" s="53"/>
+    <row customHeight="1" ht="16" r="188" s="53"/>
+    <row customHeight="1" ht="16" r="189" s="53"/>
+    <row customHeight="1" ht="16" r="190" s="53"/>
+    <row customHeight="1" ht="16" r="191" s="53"/>
+    <row customHeight="1" ht="16" r="192" s="53"/>
+    <row customHeight="1" ht="16" r="193" s="53"/>
+    <row customHeight="1" ht="16" r="194" s="53"/>
+    <row customHeight="1" ht="16" r="195" s="53"/>
+    <row customHeight="1" ht="16" r="196" s="53"/>
+    <row customHeight="1" ht="16" r="197" s="53"/>
+    <row customHeight="1" ht="16" r="198" s="53"/>
+    <row customHeight="1" ht="16" r="199" s="53"/>
+    <row customHeight="1" ht="16" r="200" s="53"/>
+    <row customHeight="1" ht="16" r="201" s="53"/>
+    <row customHeight="1" ht="16" r="202" s="53"/>
+    <row customHeight="1" ht="16" r="203" s="53"/>
+    <row customHeight="1" ht="16" r="204" s="53"/>
+    <row customHeight="1" ht="16" r="205" s="53"/>
+    <row customHeight="1" ht="16" r="206" s="53"/>
+    <row customHeight="1" ht="16" r="207" s="53"/>
+    <row customHeight="1" ht="16" r="208" s="53"/>
+    <row customHeight="1" ht="16" r="209" s="53"/>
+    <row customHeight="1" ht="16" r="210" s="53"/>
+    <row customHeight="1" ht="16" r="211" s="53"/>
+    <row customHeight="1" ht="16" r="212" s="53"/>
+    <row customHeight="1" ht="16" r="213" s="53"/>
+    <row customHeight="1" ht="16" r="214" s="53"/>
+    <row customHeight="1" ht="16" r="215" s="53"/>
+    <row customHeight="1" ht="16" r="216" s="53"/>
+    <row customHeight="1" ht="16" r="217" s="53"/>
+    <row customHeight="1" ht="16" r="218" s="53"/>
+    <row customHeight="1" ht="16" r="219" s="53"/>
+    <row customHeight="1" ht="16" r="220" s="53"/>
+    <row customHeight="1" ht="16" r="221" s="53"/>
+    <row customHeight="1" ht="16" r="222" s="53"/>
+    <row customHeight="1" ht="16" r="223" s="53"/>
+    <row customHeight="1" ht="16" r="224" s="53"/>
+    <row customHeight="1" ht="16" r="225" s="53"/>
+    <row customHeight="1" ht="16" r="226" s="53"/>
+    <row customHeight="1" ht="16" r="227" s="53"/>
+    <row customHeight="1" ht="16" r="228" s="53"/>
+    <row customHeight="1" ht="16" r="229" s="53"/>
+    <row customHeight="1" ht="16" r="230" s="53"/>
+    <row customHeight="1" ht="16" r="231" s="53"/>
+    <row customHeight="1" ht="16" r="232" s="53"/>
+    <row customHeight="1" ht="16" r="233" s="53"/>
+    <row customHeight="1" ht="16" r="234" s="53"/>
+    <row customHeight="1" ht="16" r="235" s="53"/>
+    <row customHeight="1" ht="16" r="236" s="53"/>
+    <row customHeight="1" ht="16" r="237" s="53"/>
+    <row customHeight="1" ht="16" r="238" s="53"/>
+    <row customHeight="1" ht="16" r="239" s="53"/>
+    <row customHeight="1" ht="16" r="240" s="53"/>
+    <row customHeight="1" ht="16" r="241" s="53"/>
+    <row customHeight="1" ht="16" r="242" s="53"/>
+    <row customHeight="1" ht="16" r="243" s="53"/>
+    <row customHeight="1" ht="16" r="244" s="53"/>
+    <row customHeight="1" ht="16" r="245" s="53"/>
+    <row customHeight="1" ht="16" r="246" s="53"/>
+    <row customHeight="1" ht="16" r="247" s="53"/>
+    <row customHeight="1" ht="16" r="248" s="53"/>
+    <row customHeight="1" ht="16" r="249" s="53"/>
+    <row customHeight="1" ht="16" r="250" s="53"/>
+    <row customHeight="1" ht="16" r="251" s="53"/>
+    <row customHeight="1" ht="16" r="252" s="53"/>
+    <row customHeight="1" ht="16" r="253" s="53"/>
+    <row customHeight="1" ht="16" r="254" s="53"/>
+    <row customHeight="1" ht="16" r="255" s="53"/>
+    <row customHeight="1" ht="16" r="256" s="53"/>
+    <row customHeight="1" ht="16" r="257" s="53"/>
+    <row customHeight="1" ht="16" r="258" s="53"/>
+    <row customHeight="1" ht="16" r="259" s="53"/>
+    <row customHeight="1" ht="16" r="260" s="53"/>
+    <row customHeight="1" ht="16" r="261" s="53"/>
+    <row customHeight="1" ht="16" r="262" s="53"/>
   </sheetData>
   <autoFilter ref="A2:F61"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -4885,17 +4889,17 @@
   <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -4918,7 +4922,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>区域</t>
@@ -5004,7 +5008,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5047,7 +5051,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5092,7 +5096,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5129,7 +5133,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5174,7 +5178,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5213,7 +5217,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5250,7 +5254,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5279,7 +5283,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5318,7 +5322,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5355,7 +5359,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5392,7 +5396,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5431,7 +5435,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5468,7 +5472,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5495,7 +5499,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="10" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5523,7 +5527,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5551,7 +5555,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5579,7 +5583,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5609,7 +5613,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5639,7 +5643,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5675,7 +5679,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5703,7 +5707,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5733,7 +5737,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5771,7 +5775,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5801,7 +5805,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5833,7 +5837,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5867,7 +5871,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5899,7 +5903,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5927,7 +5931,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5963,7 +5967,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5990,7 +5994,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="10" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6022,7 +6026,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6054,7 +6058,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6079,7 +6083,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6109,7 +6113,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6139,7 +6143,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6173,7 +6177,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6203,7 +6207,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6231,7 +6235,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6259,7 +6263,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6287,7 +6291,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6315,7 +6319,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6343,7 +6347,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6371,7 +6375,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6399,7 +6403,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6427,7 +6431,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6465,7 +6469,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6495,7 +6499,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6531,7 +6535,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6565,7 +6569,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6601,7 +6605,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6633,7 +6637,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -7281,7 +7285,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -7294,17 +7298,17 @@
   <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -7327,7 +7331,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>区域</t>
@@ -7413,7 +7417,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7459,7 +7463,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7496,7 +7500,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7542,7 +7546,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7588,7 +7592,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7636,7 +7640,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7673,7 +7677,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7710,7 +7714,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7758,7 +7762,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7804,7 +7808,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7841,7 +7845,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7878,7 +7882,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7924,7 +7928,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7952,7 +7956,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -7980,7 +7984,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8008,7 +8012,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8036,7 +8040,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8064,7 +8068,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8092,7 +8096,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8120,7 +8124,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8148,7 +8152,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8176,7 +8180,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8204,7 +8208,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8232,7 +8236,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8260,7 +8264,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8288,7 +8292,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8318,7 +8322,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8346,7 +8350,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8374,7 +8378,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8402,7 +8406,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8430,7 +8434,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8458,7 +8462,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8486,7 +8490,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8516,7 +8520,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8544,7 +8548,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8572,7 +8576,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8600,7 +8604,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8628,7 +8632,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8658,7 +8662,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8690,7 +8694,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8718,7 +8722,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8746,7 +8750,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8774,7 +8778,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8802,7 +8806,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8830,7 +8834,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8862,7 +8866,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8894,7 +8898,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9570,7 +9574,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -9581,16 +9585,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
@@ -9600,7 +9604,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -9645,7 +9649,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9691,7 +9695,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9736,7 +9740,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9785,7 +9789,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9834,7 +9838,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9876,7 +9880,7 @@
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="35" t="n"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9911,7 +9915,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9951,7 +9955,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9987,7 +9991,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10023,7 +10027,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10059,7 +10063,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10100,7 +10104,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10131,7 +10135,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10153,7 +10157,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10170,7 +10174,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10187,7 +10191,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10209,7 +10213,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10226,7 +10230,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10244,7 +10248,7 @@
       </c>
       <c r="D20" s="39" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10266,7 +10270,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10288,7 +10292,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10310,7 +10314,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10332,7 +10336,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10350,7 +10354,7 @@
       </c>
       <c r="D25" s="36" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10372,7 +10376,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10394,7 +10398,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10416,7 +10420,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10438,7 +10442,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10460,7 +10464,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10482,7 +10486,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10509,7 +10513,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10531,7 +10535,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10553,7 +10557,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10575,7 +10579,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10597,7 +10601,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10619,7 +10623,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10641,7 +10645,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10658,7 +10662,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10680,7 +10684,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10698,7 +10702,7 @@
       </c>
       <c r="D41" s="46" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10720,7 +10724,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10738,7 +10742,7 @@
       </c>
       <c r="D43" s="46" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10756,7 +10760,7 @@
       </c>
       <c r="E44" s="46" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10778,7 +10782,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10800,7 +10804,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10822,7 +10826,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10844,7 +10848,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10866,7 +10870,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10889,7 +10893,7 @@
       </c>
       <c r="E50" s="49" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10911,7 +10915,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10933,7 +10937,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10955,7 +10959,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="55" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -10977,7 +10981,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="55" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10999,7 +11003,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11021,7 +11025,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11039,7 +11043,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -11050,18 +11054,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6.83203125" customWidth="1" style="23" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="23" min="2" max="2"/>
-    <col width="19.6640625" customWidth="1" style="23" min="3" max="3"/>
-    <col width="13" customWidth="1" style="23" min="4" max="4"/>
-    <col hidden="1" width="30.5" customWidth="1" style="23" min="5" max="6"/>
-    <col width="30.5" customWidth="1" style="23" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="23" min="8" max="26"/>
+    <col customWidth="1" max="1" min="1" style="23" width="6.83203125"/>
+    <col customWidth="1" max="2" min="2" style="23" width="8.83203125"/>
+    <col customWidth="1" max="3" min="3" style="23" width="19.6640625"/>
+    <col customWidth="1" max="4" min="4" style="23" width="13"/>
+    <col customWidth="1" hidden="1" max="6" min="5" style="23" width="30.5"/>
+    <col customWidth="1" max="7" min="7" style="23" width="30.5"/>
+    <col customWidth="1" max="26" min="8" style="23" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="1" s="53">
       <c r="A1" s="21" t="n"/>
       <c r="B1" s="22" t="inlineStr">
         <is>
@@ -11103,7 +11107,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="2" s="53">
       <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
@@ -11146,7 +11150,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="3" s="53">
       <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
@@ -11179,7 +11183,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="4" s="53">
       <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
@@ -11217,7 +11221,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="5" s="53">
       <c r="A5" s="24" t="n">
         <v>4</v>
       </c>
@@ -11260,7 +11264,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="6" s="53">
       <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
@@ -11293,7 +11297,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="7" s="53">
       <c r="A7" s="24" t="n">
         <v>6</v>
       </c>
@@ -11322,7 +11326,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="8" s="53">
       <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
@@ -11352,7 +11356,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="9" s="53">
       <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
@@ -11377,7 +11381,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="10" s="53">
       <c r="A10" s="24" t="n">
         <v>1</v>
       </c>
@@ -11402,7 +11406,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="11" s="53">
       <c r="A11" s="24" t="n">
         <v>2</v>
       </c>
@@ -11432,7 +11436,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="12" s="53">
       <c r="A12" s="24" t="n">
         <v>3</v>
       </c>
@@ -11457,7 +11461,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="13" s="53">
       <c r="A13" s="24" t="n">
         <v>4</v>
       </c>
@@ -11487,7 +11491,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="14" s="53">
       <c r="A14" s="24" t="n">
         <v>5</v>
       </c>
@@ -11507,7 +11511,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="15" s="53">
       <c r="A15" s="24" t="n">
         <v>6</v>
       </c>
@@ -11537,7 +11541,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="16" s="53">
       <c r="A16" s="24" t="n">
         <v>1</v>
       </c>
@@ -11562,7 +11566,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="17" s="53">
       <c r="A17" s="24" t="n">
         <v>2</v>
       </c>
@@ -11597,7 +11601,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="18" s="53">
       <c r="A18" s="24" t="n">
         <v>3</v>
       </c>
@@ -11632,7 +11636,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="19" s="53">
       <c r="A19" s="24" t="n">
         <v>4</v>
       </c>
@@ -11657,7 +11661,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="20" s="53">
       <c r="A20" s="24" t="n">
         <v>5</v>
       </c>
@@ -11687,7 +11691,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="21" s="53">
       <c r="A21" s="24" t="n">
         <v>6</v>
       </c>
@@ -11717,7 +11721,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="22" s="53">
       <c r="A22" s="24" t="n">
         <v>7</v>
       </c>
@@ -11747,7 +11751,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="23" s="53">
       <c r="A23" s="24" t="n">
         <v>8</v>
       </c>
@@ -11777,7 +11781,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="24" s="53">
       <c r="A24" s="24" t="n">
         <v>1</v>
       </c>
@@ -11807,7 +11811,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="25" s="53">
       <c r="A25" s="24" t="n">
         <v>2</v>
       </c>
@@ -11837,7 +11841,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="26" s="53">
       <c r="A26" s="24" t="n">
         <v>3</v>
       </c>
@@ -11862,7 +11866,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="27" s="53">
       <c r="A27" s="24" t="n">
         <v>4</v>
       </c>
@@ -11892,7 +11896,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="28" s="53">
       <c r="A28" s="24" t="n">
         <v>5</v>
       </c>
@@ -11922,7 +11926,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="29" s="53">
       <c r="A29" s="24" t="n">
         <v>6</v>
       </c>
@@ -11952,7 +11956,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="30" s="53">
       <c r="A30" s="24" t="n">
         <v>7</v>
       </c>
@@ -11987,7 +11991,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="31" s="53">
       <c r="A31" s="24" t="n">
         <v>8</v>
       </c>
@@ -12017,7 +12021,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="32" s="53">
       <c r="A32" s="24" t="n">
         <v>1</v>
       </c>
@@ -12047,7 +12051,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="33" s="53">
       <c r="A33" s="24" t="n">
         <v>2</v>
       </c>
@@ -12077,7 +12081,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="34" s="53">
       <c r="A34" s="24" t="n">
         <v>3</v>
       </c>
@@ -12107,7 +12111,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="35" s="53">
       <c r="A35" s="24" t="n">
         <v>4</v>
       </c>
@@ -12137,7 +12141,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="36" s="53">
       <c r="A36" s="24" t="n">
         <v>1</v>
       </c>
@@ -12167,7 +12171,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="37" s="53">
       <c r="A37" s="24" t="n">
         <v>2</v>
       </c>
@@ -12202,7 +12206,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="38" s="53">
       <c r="A38" s="24" t="n">
         <v>3</v>
       </c>
@@ -12233,6 +12237,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
report: update 2026-08-20 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46250</v>
+        <v>46254</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="D43" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发2次</t>
+          <t>累计未发2次，迟发2次</t>
         </is>
       </c>
       <c r="E43" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-22 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46254</v>
+        <v>46256</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3872,7 +3872,7 @@
       </c>
       <c r="D36" s="73" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发3次，迟发1次</t>
         </is>
       </c>
       <c r="E36" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-23 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="D43" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发2次</t>
+          <t>累计未发2次，迟发3次</t>
         </is>
       </c>
       <c r="E43" s="69" t="n"/>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="D58" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="E58" s="69" t="n"/>
@@ -4538,7 +4538,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D60" s="68" t="n"/>
+      <c r="D60" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E60" s="69" t="n"/>
       <c r="F60" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-08-24 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="D55" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-25 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="D6" s="68" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发4次</t>
         </is>
       </c>
       <c r="E6" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-26 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="D48" s="71" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E48" s="69" t="n"/>
@@ -4453,7 +4453,7 @@
       </c>
       <c r="D57" s="68" t="inlineStr">
         <is>
-          <t>累计未发4次</t>
+          <t>累计未发5次</t>
         </is>
       </c>
       <c r="E57" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-28 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3467,7 +3467,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D21" s="73" t="n"/>
+      <c r="D21" s="73" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E21" s="69" t="n"/>
       <c r="F21" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-08-29 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="D6" s="68" t="inlineStr">
         <is>
-          <t>累计未发4次</t>
+          <t>累计未发5次</t>
         </is>
       </c>
       <c r="E6" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-08-30 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="D19" s="68" t="inlineStr">
         <is>
-          <t>累计未发3次</t>
+          <t>累计未发4次</t>
         </is>
       </c>
       <c r="E19" s="69" t="n"/>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="D30" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发3次</t>
+          <t>累计未发2次，迟发3次</t>
         </is>
       </c>
       <c r="E30" s="69" t="n"/>
@@ -3849,7 +3849,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D35" s="71" t="n"/>
+      <c r="D35" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E35" s="69" t="n"/>
       <c r="F35" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-09-03 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46264</v>
+        <v>46268</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2947,7 +2947,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D7" s="70" t="n"/>
+      <c r="D7" s="70" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E7" s="69" t="n"/>
       <c r="F7" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-09-05 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D30" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发3次</t>
+          <t>累计未发3次，迟发3次</t>
         </is>
       </c>
       <c r="E30" s="69" t="n"/>

</xml_diff>